<commit_message>
Fix build and push updated site
</commit_message>
<xml_diff>
--- a/estimates_PS2025.xlsx
+++ b/estimates_PS2025.xlsx
@@ -8,14 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\GitHub\tibor-pal.github.io\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22F2597C-608C-4CED-8C74-F252BECE5AC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A119400-E635-4BD9-B063-3F5F1AB07DC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{898E4DB8-E74C-49BD-9493-76D0D230C2FB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="4" r:id="rId2"/>
-    <sheet name="info_READ IT" sheetId="3" r:id="rId3"/>
+    <sheet name="info_READ IT" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -16699,3926 +16698,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06608B4E-EAA6-452E-B862-B69EDA33F1C2}">
-  <dimension ref="A1:IZ5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:260" x14ac:dyDescent="0.25">
-      <c r="A1">
-        <v>9.0445374117341104E-2</v>
-      </c>
-      <c r="B1">
-        <v>6.8774425146596693E-2</v>
-      </c>
-      <c r="C1">
-        <v>7.1188816541932695E-2</v>
-      </c>
-      <c r="D1">
-        <v>7.3202624204753403E-2</v>
-      </c>
-      <c r="E1">
-        <v>7.4697687840799901E-2</v>
-      </c>
-      <c r="F1">
-        <v>7.5856271099876693E-2</v>
-      </c>
-      <c r="G1">
-        <v>7.6976002482605804E-2</v>
-      </c>
-      <c r="H1">
-        <v>7.7942761067055596E-2</v>
-      </c>
-      <c r="I1">
-        <v>7.9150876900161204E-2</v>
-      </c>
-      <c r="J1">
-        <v>8.0274953069030902E-2</v>
-      </c>
-      <c r="K1">
-        <v>8.1309791980819196E-2</v>
-      </c>
-      <c r="L1">
-        <v>8.1767797152881697E-2</v>
-      </c>
-      <c r="M1">
-        <v>8.2391330826118103E-2</v>
-      </c>
-      <c r="N1">
-        <v>8.2481870045831199E-2</v>
-      </c>
-      <c r="O1">
-        <v>8.2565236916010407E-2</v>
-      </c>
-      <c r="P1">
-        <v>8.2412498494380398E-2</v>
-      </c>
-      <c r="Q1">
-        <v>8.2643071224551695E-2</v>
-      </c>
-      <c r="R1">
-        <v>8.2232564830626007E-2</v>
-      </c>
-      <c r="S1">
-        <v>8.1770354900772099E-2</v>
-      </c>
-      <c r="T1">
-        <v>8.0835816163277299E-2</v>
-      </c>
-      <c r="U1">
-        <v>7.94747953087383E-2</v>
-      </c>
-      <c r="V1">
-        <v>7.7730253753580003E-2</v>
-      </c>
-      <c r="W1">
-        <v>7.6536104294358406E-2</v>
-      </c>
-      <c r="X1">
-        <v>7.5594104239680507E-2</v>
-      </c>
-      <c r="Y1">
-        <v>7.4878785298722605E-2</v>
-      </c>
-      <c r="Z1">
-        <v>0.114161695341829</v>
-      </c>
-      <c r="AA1">
-        <v>0.109166339459949</v>
-      </c>
-      <c r="AB1">
-        <v>0.10501778554728899</v>
-      </c>
-      <c r="AC1">
-        <v>0.101702981983993</v>
-      </c>
-      <c r="AD1">
-        <v>9.8179203290138198E-2</v>
-      </c>
-      <c r="AE1">
-        <v>9.4772318354776494E-2</v>
-      </c>
-      <c r="AF1">
-        <v>9.2045046750306905E-2</v>
-      </c>
-      <c r="AG1">
-        <v>9.0080034176316201E-2</v>
-      </c>
-      <c r="AH1">
-        <v>8.8082994138567502E-2</v>
-      </c>
-      <c r="AI1">
-        <v>8.6710039640746195E-2</v>
-      </c>
-      <c r="AJ1">
-        <v>8.5645034509310894E-2</v>
-      </c>
-      <c r="AK1">
-        <v>8.5387876190850698E-2</v>
-      </c>
-      <c r="AL1">
-        <v>8.5660187613700103E-2</v>
-      </c>
-      <c r="AM1">
-        <v>8.6264715096007499E-2</v>
-      </c>
-      <c r="AN1">
-        <v>8.6791072738770597E-2</v>
-      </c>
-      <c r="AO1">
-        <v>8.8226561115741897E-2</v>
-      </c>
-      <c r="AP1">
-        <v>8.8620065311926705E-2</v>
-      </c>
-      <c r="AQ1">
-        <v>8.9124662198983198E-2</v>
-      </c>
-      <c r="AR1">
-        <v>8.9563787838392805E-2</v>
-      </c>
-      <c r="AS1">
-        <v>7.8550437846002796E-2</v>
-      </c>
-      <c r="AT1">
-        <v>7.9501483508608195E-2</v>
-      </c>
-      <c r="AU1">
-        <v>8.3594668860570501E-2</v>
-      </c>
-      <c r="AV1">
-        <v>8.3434010513750503E-2</v>
-      </c>
-      <c r="AW1">
-        <v>8.2823232113683795E-2</v>
-      </c>
-      <c r="AX1">
-        <v>8.1532970974785998E-2</v>
-      </c>
-      <c r="AY1">
-        <v>8.0303469262417798E-2</v>
-      </c>
-      <c r="AZ1">
-        <v>7.9856034696382597E-2</v>
-      </c>
-      <c r="BA1">
-        <v>7.9424631725675404E-2</v>
-      </c>
-      <c r="BB1">
-        <v>7.9801860578208594E-2</v>
-      </c>
-      <c r="BC1">
-        <v>8.0432796174060295E-2</v>
-      </c>
-      <c r="BD1">
-        <v>8.1826004003687794E-2</v>
-      </c>
-      <c r="BE1">
-        <v>8.37166915321709E-2</v>
-      </c>
-      <c r="BF1">
-        <v>8.6701138175599296E-2</v>
-      </c>
-      <c r="BG1">
-        <v>9.0052517747227501E-2</v>
-      </c>
-      <c r="BH1">
-        <v>9.2298706771706596E-2</v>
-      </c>
-      <c r="BI1">
-        <v>9.4173440835661995E-2</v>
-      </c>
-      <c r="BJ1">
-        <v>9.5084222381932204E-2</v>
-      </c>
-      <c r="BK1">
-        <v>7.9662667677503907E-2</v>
-      </c>
-      <c r="BL1">
-        <v>8.1581380891965399E-2</v>
-      </c>
-      <c r="BM1">
-        <v>8.3453073471340802E-2</v>
-      </c>
-      <c r="BN1">
-        <v>8.4756058471633006E-2</v>
-      </c>
-      <c r="BO1">
-        <v>8.5579495096101396E-2</v>
-      </c>
-      <c r="BP1">
-        <v>8.5837489114667098E-2</v>
-      </c>
-      <c r="BQ1">
-        <v>8.6441780559886397E-2</v>
-      </c>
-      <c r="BR1">
-        <v>8.7448172085484194E-2</v>
-      </c>
-      <c r="BS1">
-        <v>8.6859851733783897E-2</v>
-      </c>
-      <c r="BT1">
-        <v>8.5973436367112702E-2</v>
-      </c>
-      <c r="BU1">
-        <v>8.5090438852318803E-2</v>
-      </c>
-      <c r="BV1">
-        <v>0.101629950160303</v>
-      </c>
-      <c r="BW1">
-        <v>0.100084199398926</v>
-      </c>
-      <c r="BX1">
-        <v>9.8741952284549794E-2</v>
-      </c>
-      <c r="BY1">
-        <v>9.7871329358345097E-2</v>
-      </c>
-      <c r="BZ1">
-        <v>9.7315197170671594E-2</v>
-      </c>
-      <c r="CA1">
-        <v>9.8579500806110304E-2</v>
-      </c>
-      <c r="CB1">
-        <v>0.100556698352583</v>
-      </c>
-      <c r="CC1">
-        <v>0.100949140916579</v>
-      </c>
-      <c r="CD1">
-        <v>0.10056679505701301</v>
-      </c>
-      <c r="CE1">
-        <v>8.4074955557960296E-2</v>
-      </c>
-      <c r="CF1">
-        <v>8.5284890603212399E-2</v>
-      </c>
-      <c r="CG1">
-        <v>8.7413610746257503E-2</v>
-      </c>
-      <c r="CH1">
-        <v>6.1834588953356501E-2</v>
-      </c>
-      <c r="CI1">
-        <v>6.5129320560502801E-2</v>
-      </c>
-      <c r="CJ1">
-        <v>6.8736619513303093E-2</v>
-      </c>
-      <c r="CK1">
-        <v>7.2598379812860506E-2</v>
-      </c>
-      <c r="CL1">
-        <v>7.6316873101567803E-2</v>
-      </c>
-      <c r="CM1">
-        <v>3.3108696364596998E-2</v>
-      </c>
-      <c r="CN1">
-        <v>3.6075219039786902E-2</v>
-      </c>
-      <c r="CO1">
-        <v>3.1407604382902701E-2</v>
-      </c>
-      <c r="CP1">
-        <v>3.41884767176759E-2</v>
-      </c>
-      <c r="CQ1">
-        <v>3.6906344148138003E-2</v>
-      </c>
-      <c r="CR1">
-        <v>3.9350097035376903E-2</v>
-      </c>
-      <c r="CS1">
-        <v>4.1638461227038501E-2</v>
-      </c>
-      <c r="CT1">
-        <v>4.4307484548915699E-2</v>
-      </c>
-      <c r="CU1">
-        <v>4.6860108507967201E-2</v>
-      </c>
-      <c r="CV1">
-        <v>4.9317455834730302E-2</v>
-      </c>
-      <c r="CW1">
-        <v>5.1545972803514202E-2</v>
-      </c>
-      <c r="CX1">
-        <v>5.3861000343945302E-2</v>
-      </c>
-      <c r="CY1">
-        <v>5.5485257289964798E-2</v>
-      </c>
-      <c r="CZ1">
-        <v>5.7706586820647998E-2</v>
-      </c>
-      <c r="DA1">
-        <v>5.9905497074500901E-2</v>
-      </c>
-      <c r="DB1">
-        <v>6.2018805097086897E-2</v>
-      </c>
-      <c r="DC1">
-        <v>6.3979056704491194E-2</v>
-      </c>
-      <c r="DD1">
-        <v>6.5821352577582606E-2</v>
-      </c>
-      <c r="DE1">
-        <v>6.7283266412504497E-2</v>
-      </c>
-      <c r="DF1">
-        <v>6.8733916051999397E-2</v>
-      </c>
-      <c r="DG1">
-        <v>6.9909547997095298E-2</v>
-      </c>
-      <c r="DH1">
-        <v>7.1059413535492402E-2</v>
-      </c>
-      <c r="DI1">
-        <v>7.1919302102888494E-2</v>
-      </c>
-      <c r="DJ1">
-        <v>7.2612406459455894E-2</v>
-      </c>
-      <c r="DK1">
-        <v>7.3473365331299903E-2</v>
-      </c>
-      <c r="DL1">
-        <v>7.4090894965952406E-2</v>
-      </c>
-      <c r="DM1">
-        <v>7.47103157051862E-2</v>
-      </c>
-      <c r="DN1">
-        <v>7.5102829509343799E-2</v>
-      </c>
-      <c r="DO1">
-        <v>7.5676346812484793E-2</v>
-      </c>
-      <c r="DP1">
-        <v>7.6454163481553095E-2</v>
-      </c>
-      <c r="DQ1">
-        <v>7.7823496838163406E-2</v>
-      </c>
-      <c r="DR1">
-        <v>7.9592399429392405E-2</v>
-      </c>
-      <c r="DS1">
-        <v>8.1223444458114802E-2</v>
-      </c>
-      <c r="DT1">
-        <v>8.2965909940325697E-2</v>
-      </c>
-      <c r="DU1">
-        <v>8.4464662225018902E-2</v>
-      </c>
-      <c r="DV1">
-        <v>8.5661134772891001E-2</v>
-      </c>
-      <c r="DW1">
-        <v>8.6721360168553696E-2</v>
-      </c>
-      <c r="DX1">
-        <v>8.7545068791967703E-2</v>
-      </c>
-      <c r="DY1">
-        <v>8.8050735826225093E-2</v>
-      </c>
-      <c r="DZ1">
-        <v>8.8765630486024497E-2</v>
-      </c>
-      <c r="EA1">
-        <v>8.9608946993323502E-2</v>
-      </c>
-      <c r="EB1">
-        <v>8.9998155171779504E-2</v>
-      </c>
-      <c r="EC1">
-        <v>9.0571165682299698E-2</v>
-      </c>
-      <c r="ED1">
-        <v>9.1004924981950702E-2</v>
-      </c>
-      <c r="EE1">
-        <v>9.0897640486387404E-2</v>
-      </c>
-      <c r="EF1">
-        <v>9.0898558495376203E-2</v>
-      </c>
-      <c r="EG1">
-        <v>9.0601631362193902E-2</v>
-      </c>
-      <c r="EH1">
-        <v>9.0582185899649406E-2</v>
-      </c>
-      <c r="EI1">
-        <v>9.0851578659721197E-2</v>
-      </c>
-      <c r="EJ1">
-        <v>9.1104540548787402E-2</v>
-      </c>
-      <c r="EK1">
-        <v>9.1301763670682101E-2</v>
-      </c>
-      <c r="EL1">
-        <v>9.1583763200018001E-2</v>
-      </c>
-      <c r="EM1">
-        <v>9.1162108693509006E-2</v>
-      </c>
-      <c r="EN1">
-        <v>9.0730043507647296E-2</v>
-      </c>
-      <c r="EO1">
-        <v>9.0301355810577993E-2</v>
-      </c>
-      <c r="EP1">
-        <v>9.0560237342266106E-2</v>
-      </c>
-      <c r="EQ1">
-        <v>8.9795110053120006E-2</v>
-      </c>
-      <c r="ER1">
-        <v>0.10133108859859</v>
-      </c>
-      <c r="ES1">
-        <v>9.9383955911313507E-2</v>
-      </c>
-      <c r="ET1">
-        <v>9.7781701753864803E-2</v>
-      </c>
-      <c r="EU1">
-        <v>9.6426704980631897E-2</v>
-      </c>
-      <c r="EV1">
-        <v>9.5070858949086595E-2</v>
-      </c>
-      <c r="EW1">
-        <v>9.3495224235628296E-2</v>
-      </c>
-      <c r="EX1">
-        <v>9.2186469461295703E-2</v>
-      </c>
-      <c r="EY1">
-        <v>9.1149227192112006E-2</v>
-      </c>
-      <c r="EZ1">
-        <v>9.0065690444412302E-2</v>
-      </c>
-      <c r="FA1">
-        <v>8.8778332323100201E-2</v>
-      </c>
-      <c r="FB1">
-        <v>8.80067074896526E-2</v>
-      </c>
-      <c r="FC1">
-        <v>8.7337858798344201E-2</v>
-      </c>
-      <c r="FD1">
-        <v>8.6732203900841104E-2</v>
-      </c>
-      <c r="FE1">
-        <v>8.6360184738031698E-2</v>
-      </c>
-      <c r="FF1">
-        <v>8.6650886859119897E-2</v>
-      </c>
-      <c r="FG1">
-        <v>8.6282504583214598E-2</v>
-      </c>
-      <c r="FH1">
-        <v>8.7256078116678196E-2</v>
-      </c>
-      <c r="FI1">
-        <v>8.8414335470980696E-2</v>
-      </c>
-      <c r="FJ1">
-        <v>8.9393113022620596E-2</v>
-      </c>
-      <c r="FK1">
-        <v>9.0334816463102E-2</v>
-      </c>
-      <c r="FL1">
-        <v>9.1332447787331905E-2</v>
-      </c>
-      <c r="FM1">
-        <v>9.2192243284134806E-2</v>
-      </c>
-      <c r="FN1">
-        <v>9.3369827595381497E-2</v>
-      </c>
-      <c r="FO1">
-        <v>9.4325612679757101E-2</v>
-      </c>
-      <c r="FP1">
-        <v>9.4576363206739705E-2</v>
-      </c>
-      <c r="FQ1">
-        <v>9.4466664041967296E-2</v>
-      </c>
-      <c r="FR1">
-        <v>9.4399978020285505E-2</v>
-      </c>
-      <c r="FS1">
-        <v>9.4248890882717096E-2</v>
-      </c>
-      <c r="FT1">
-        <v>9.4026171490874999E-2</v>
-      </c>
-      <c r="FU1">
-        <v>9.3486948547244805E-2</v>
-      </c>
-      <c r="FV1">
-        <v>9.2707224517624198E-2</v>
-      </c>
-      <c r="FW1">
-        <v>9.4564590649703503E-2</v>
-      </c>
-      <c r="FX1">
-        <v>9.3306371512319894E-2</v>
-      </c>
-      <c r="FY1">
-        <v>9.2625272872836603E-2</v>
-      </c>
-      <c r="FZ1">
-        <v>9.12800825271919E-2</v>
-      </c>
-      <c r="GA1">
-        <v>9.0443303293523597E-2</v>
-      </c>
-      <c r="GB1">
-        <v>9.3789630574326502E-2</v>
-      </c>
-      <c r="GC1">
-        <v>9.2179946063148499E-2</v>
-      </c>
-      <c r="GD1">
-        <v>9.13982144853724E-2</v>
-      </c>
-      <c r="GE1">
-        <v>9.26024636143047E-2</v>
-      </c>
-      <c r="GF1">
-        <v>9.1662355529595396E-2</v>
-      </c>
-      <c r="GG1">
-        <v>9.0743937496232205E-2</v>
-      </c>
-      <c r="GH1">
-        <v>9.0537243643496801E-2</v>
-      </c>
-      <c r="GI1">
-        <v>9.0214608338500604E-2</v>
-      </c>
-      <c r="GJ1">
-        <v>9.0497025916028803E-2</v>
-      </c>
-      <c r="GK1">
-        <v>5.0334008386115299E-2</v>
-      </c>
-      <c r="GL1">
-        <v>5.3123136271060897E-2</v>
-      </c>
-      <c r="GM1">
-        <v>5.6371871721573902E-2</v>
-      </c>
-      <c r="GN1">
-        <v>5.9756526253782902E-2</v>
-      </c>
-      <c r="GO1">
-        <v>6.2773816279892106E-2</v>
-      </c>
-      <c r="GP1">
-        <v>6.4357130949793798E-2</v>
-      </c>
-      <c r="GQ1">
-        <v>6.7083588086327098E-2</v>
-      </c>
-      <c r="GR1">
-        <v>6.9450717097172598E-2</v>
-      </c>
-      <c r="GS1">
-        <v>7.1853545360918203E-2</v>
-      </c>
-      <c r="GT1">
-        <v>7.4402601535044105E-2</v>
-      </c>
-      <c r="GU1">
-        <v>7.6781115981318204E-2</v>
-      </c>
-      <c r="GV1">
-        <v>7.9033660838019507E-2</v>
-      </c>
-      <c r="GW1">
-        <v>8.1141176825042502E-2</v>
-      </c>
-      <c r="GX1">
-        <v>8.2980459385771102E-2</v>
-      </c>
-      <c r="GY1">
-        <v>8.4522393121375897E-2</v>
-      </c>
-      <c r="GZ1">
-        <v>8.6517938817153001E-2</v>
-      </c>
-      <c r="HA1">
-        <v>8.8424686341394901E-2</v>
-      </c>
-      <c r="HB1">
-        <v>8.9988758534976301E-2</v>
-      </c>
-      <c r="HC1">
-        <v>9.2473867250927197E-2</v>
-      </c>
-      <c r="HD1">
-        <v>9.3926238913541599E-2</v>
-      </c>
-      <c r="HE1">
-        <v>9.5014334757685198E-2</v>
-      </c>
-      <c r="HF1">
-        <v>9.74309717206749E-2</v>
-      </c>
-      <c r="HG1">
-        <v>9.8343823789619006E-2</v>
-      </c>
-      <c r="HH1">
-        <v>9.8728189641100597E-2</v>
-      </c>
-      <c r="HI1">
-        <v>9.9353920633906995E-2</v>
-      </c>
-      <c r="HJ1">
-        <v>9.9421650965629396E-2</v>
-      </c>
-      <c r="HK1">
-        <v>9.9221488468815996E-2</v>
-      </c>
-      <c r="HL1">
-        <v>9.9277536867103403E-2</v>
-      </c>
-      <c r="HM1">
-        <v>9.9508638469980606E-2</v>
-      </c>
-      <c r="HN1">
-        <v>9.9600567724879505E-2</v>
-      </c>
-      <c r="HO1">
-        <v>9.9837210481090094E-2</v>
-      </c>
-      <c r="HP1">
-        <v>0.10018094816878501</v>
-      </c>
-      <c r="HQ1">
-        <v>0.100311287938882</v>
-      </c>
-      <c r="HR1">
-        <v>0.100301600043721</v>
-      </c>
-      <c r="HS1">
-        <v>0.100568370239373</v>
-      </c>
-      <c r="HT1">
-        <v>0.10025716771026399</v>
-      </c>
-      <c r="HU1">
-        <v>9.9452004487817505E-2</v>
-      </c>
-      <c r="HV1">
-        <v>9.8469554975313803E-2</v>
-      </c>
-      <c r="HW1">
-        <v>9.7479375722934095E-2</v>
-      </c>
-      <c r="HX1">
-        <v>9.7912776473394594E-2</v>
-      </c>
-      <c r="HY1">
-        <v>9.7265236686170403E-2</v>
-      </c>
-      <c r="HZ1">
-        <v>9.6583744675247205E-2</v>
-      </c>
-      <c r="IA1">
-        <v>9.5747170680535496E-2</v>
-      </c>
-      <c r="IB1">
-        <v>9.4469307133330294E-2</v>
-      </c>
-      <c r="IC1">
-        <v>9.3348413968896607E-2</v>
-      </c>
-      <c r="ID1">
-        <v>9.3462202517938395E-2</v>
-      </c>
-      <c r="IE1">
-        <v>1.7092691606898101E-2</v>
-      </c>
-      <c r="IF1">
-        <v>1.93357889476206E-2</v>
-      </c>
-      <c r="IG1">
-        <v>2.1698790942874299E-2</v>
-      </c>
-      <c r="IH1">
-        <v>2.4148633245539501E-2</v>
-      </c>
-      <c r="II1">
-        <v>2.6640916929269998E-2</v>
-      </c>
-      <c r="IJ1">
-        <v>2.9174696935404299E-2</v>
-      </c>
-      <c r="IK1">
-        <v>3.1673716246914903E-2</v>
-      </c>
-      <c r="IL1">
-        <v>3.4227650344732803E-2</v>
-      </c>
-      <c r="IM1">
-        <v>3.6843992394557802E-2</v>
-      </c>
-      <c r="IN1">
-        <v>3.93912778693771E-2</v>
-      </c>
-      <c r="IO1">
-        <v>4.1893914677098798E-2</v>
-      </c>
-      <c r="IP1">
-        <v>4.4336008301389701E-2</v>
-      </c>
-      <c r="IQ1">
-        <v>4.6680302051140002E-2</v>
-      </c>
-      <c r="IR1">
-        <v>5.1819545409306299E-2</v>
-      </c>
-      <c r="IS1">
-        <v>5.3749117018008899E-2</v>
-      </c>
-      <c r="IT1">
-        <v>5.5738161497399401E-2</v>
-      </c>
-      <c r="IU1">
-        <v>5.7561510414593599E-2</v>
-      </c>
-      <c r="IV1">
-        <v>5.91186719210781E-2</v>
-      </c>
-      <c r="IW1">
-        <v>6.0780028909221899E-2</v>
-      </c>
-      <c r="IX1">
-        <v>6.2543124429238803E-2</v>
-      </c>
-      <c r="IY1">
-        <v>6.40023839309041E-2</v>
-      </c>
-      <c r="IZ1">
-        <v>6.5335014123811597E-2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:260" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>8.6315323395899105E-2</v>
-      </c>
-      <c r="B2">
-        <v>5.43578129298804E-2</v>
-      </c>
-      <c r="C2">
-        <v>5.9700287390098701E-2</v>
-      </c>
-      <c r="D2">
-        <v>6.4075652663236907E-2</v>
-      </c>
-      <c r="E2">
-        <v>6.3001388504335606E-2</v>
-      </c>
-      <c r="F2">
-        <v>6.4698617689827806E-2</v>
-      </c>
-      <c r="G2">
-        <v>6.6446970798135496E-2</v>
-      </c>
-      <c r="H2">
-        <v>6.7778950474035995E-2</v>
-      </c>
-      <c r="I2">
-        <v>6.8550956255012604E-2</v>
-      </c>
-      <c r="J2">
-        <v>7.0990271821141093E-2</v>
-      </c>
-      <c r="K2">
-        <v>7.3272820064957597E-2</v>
-      </c>
-      <c r="L2">
-        <v>7.3263090274785794E-2</v>
-      </c>
-      <c r="M2">
-        <v>7.4104070362088506E-2</v>
-      </c>
-      <c r="N2">
-        <v>7.2942848256478995E-2</v>
-      </c>
-      <c r="O2">
-        <v>7.5204824639873505E-2</v>
-      </c>
-      <c r="P2">
-        <v>7.2826836347208296E-2</v>
-      </c>
-      <c r="Q2">
-        <v>7.2336884838039101E-2</v>
-      </c>
-      <c r="R2">
-        <v>6.9236786045212606E-2</v>
-      </c>
-      <c r="S2">
-        <v>6.7791023124460906E-2</v>
-      </c>
-      <c r="T2">
-        <v>6.3225347659501899E-2</v>
-      </c>
-      <c r="U2">
-        <v>5.7760150607457997E-2</v>
-      </c>
-      <c r="V2">
-        <v>5.1780204243870101E-2</v>
-      </c>
-      <c r="W2">
-        <v>4.8476931989371697E-2</v>
-      </c>
-      <c r="X2">
-        <v>4.6223617525353401E-2</v>
-      </c>
-      <c r="Y2">
-        <v>4.4573188400741398E-2</v>
-      </c>
-      <c r="Z2">
-        <v>6.6183853296252801E-2</v>
-      </c>
-      <c r="AA2">
-        <v>6.17803480418498E-2</v>
-      </c>
-      <c r="AB2">
-        <v>5.858093984519E-2</v>
-      </c>
-      <c r="AC2">
-        <v>5.64976340733934E-2</v>
-      </c>
-      <c r="AD2">
-        <v>5.3663937756868098E-2</v>
-      </c>
-      <c r="AE2">
-        <v>5.07162164336128E-2</v>
-      </c>
-      <c r="AF2">
-        <v>4.8756042000870602E-2</v>
-      </c>
-      <c r="AG2">
-        <v>4.7829167106566997E-2</v>
-      </c>
-      <c r="AH2">
-        <v>4.6621532407026302E-2</v>
-      </c>
-      <c r="AI2">
-        <v>4.6226524317497401E-2</v>
-      </c>
-      <c r="AJ2">
-        <v>4.6168616740062299E-2</v>
-      </c>
-      <c r="AK2">
-        <v>4.7339020388491797E-2</v>
-      </c>
-      <c r="AL2">
-        <v>4.9377801864340098E-2</v>
-      </c>
-      <c r="AM2">
-        <v>5.2045968142750303E-2</v>
-      </c>
-      <c r="AN2">
-        <v>5.4579764082719397E-2</v>
-      </c>
-      <c r="AO2">
-        <v>5.9300949168192403E-2</v>
-      </c>
-      <c r="AP2">
-        <v>6.1639592491604403E-2</v>
-      </c>
-      <c r="AQ2">
-        <v>6.4148540209668994E-2</v>
-      </c>
-      <c r="AR2">
-        <v>6.4331704761572406E-2</v>
-      </c>
-      <c r="AS2">
-        <v>5.76104154281026E-2</v>
-      </c>
-      <c r="AT2">
-        <v>5.9692506748383403E-2</v>
-      </c>
-      <c r="AU2">
-        <v>7.0066283068105195E-2</v>
-      </c>
-      <c r="AV2">
-        <v>6.8720242794238606E-2</v>
-      </c>
-      <c r="AW2">
-        <v>7.3135503950345904E-2</v>
-      </c>
-      <c r="AX2">
-        <v>6.6775433023509606E-2</v>
-      </c>
-      <c r="AY2">
-        <v>6.1568192775934998E-2</v>
-      </c>
-      <c r="AZ2">
-        <v>5.9474404641438897E-2</v>
-      </c>
-      <c r="BA2">
-        <v>5.7632937890406702E-2</v>
-      </c>
-      <c r="BB2">
-        <v>5.8226614736304999E-2</v>
-      </c>
-      <c r="BC2">
-        <v>5.95880102141454E-2</v>
-      </c>
-      <c r="BD2">
-        <v>6.3310590145066903E-2</v>
-      </c>
-      <c r="BE2">
-        <v>6.8988456268097201E-2</v>
-      </c>
-      <c r="BF2">
-        <v>7.2771543393024496E-2</v>
-      </c>
-      <c r="BG2">
-        <v>6.6970042655543904E-2</v>
-      </c>
-      <c r="BH2">
-        <v>7.4946362861918095E-2</v>
-      </c>
-      <c r="BI2">
-        <v>8.27615676847233E-2</v>
-      </c>
-      <c r="BJ2">
-        <v>8.7649122728523196E-2</v>
-      </c>
-      <c r="BK2">
-        <v>7.4829136294151402E-2</v>
-      </c>
-      <c r="BL2">
-        <v>7.9343069984861694E-2</v>
-      </c>
-      <c r="BM2">
-        <v>8.4159510640129401E-2</v>
-      </c>
-      <c r="BN2">
-        <v>8.9571117497215302E-2</v>
-      </c>
-      <c r="BO2">
-        <v>9.1409040190799207E-2</v>
-      </c>
-      <c r="BP2">
-        <v>9.0374173539135794E-2</v>
-      </c>
-      <c r="BQ2">
-        <v>8.6117301737632101E-2</v>
-      </c>
-      <c r="BR2">
-        <v>8.8810621116152497E-2</v>
-      </c>
-      <c r="BS2">
-        <v>8.3295962340667801E-2</v>
-      </c>
-      <c r="BT2">
-        <v>7.9208294313581604E-2</v>
-      </c>
-      <c r="BU2">
-        <v>7.4492830343077396E-2</v>
-      </c>
-      <c r="BV2">
-        <v>9.04694539892692E-2</v>
-      </c>
-      <c r="BW2">
-        <v>8.7654341019750795E-2</v>
-      </c>
-      <c r="BX2">
-        <v>8.5391429857317097E-2</v>
-      </c>
-      <c r="BY2">
-        <v>8.4719997674556097E-2</v>
-      </c>
-      <c r="BZ2">
-        <v>8.5028642930265796E-2</v>
-      </c>
-      <c r="CA2">
-        <v>9.2645748129357705E-2</v>
-      </c>
-      <c r="CB2">
-        <v>0.10147467107812901</v>
-      </c>
-      <c r="CC2">
-        <v>0.10857978530047099</v>
-      </c>
-      <c r="CD2">
-        <v>0.108982786848349</v>
-      </c>
-      <c r="CE2">
-        <v>7.7430644450914896E-2</v>
-      </c>
-      <c r="CF2">
-        <v>8.1019499432693196E-2</v>
-      </c>
-      <c r="CG2">
-        <v>8.8038989126317302E-2</v>
-      </c>
-      <c r="CH2">
-        <v>3.8730956751346003E-2</v>
-      </c>
-      <c r="CI2">
-        <v>4.2001768642616302E-2</v>
-      </c>
-      <c r="CJ2">
-        <v>4.92245868298287E-2</v>
-      </c>
-      <c r="CK2">
-        <v>4.7004196791116101E-2</v>
-      </c>
-      <c r="CL2">
-        <v>5.5006003698797497E-2</v>
-      </c>
-      <c r="CM2">
-        <v>3.5889552675530498E-2</v>
-      </c>
-      <c r="CN2">
-        <v>4.0337291769883002E-2</v>
-      </c>
-      <c r="CO2">
-        <v>3.5954797912130798E-2</v>
-      </c>
-      <c r="CP2">
-        <v>3.8144198697635801E-2</v>
-      </c>
-      <c r="CQ2">
-        <v>4.1094730453337301E-2</v>
-      </c>
-      <c r="CR2">
-        <v>4.1585851922658998E-2</v>
-      </c>
-      <c r="CS2">
-        <v>4.1910513143627398E-2</v>
-      </c>
-      <c r="CT2">
-        <v>4.4751395128633097E-2</v>
-      </c>
-      <c r="CU2">
-        <v>4.5882622780727501E-2</v>
-      </c>
-      <c r="CV2">
-        <v>4.82485681607994E-2</v>
-      </c>
-      <c r="CW2">
-        <v>4.9795216941308403E-2</v>
-      </c>
-      <c r="CX2">
-        <v>5.2055882588634098E-2</v>
-      </c>
-      <c r="CY2">
-        <v>5.22143794047965E-2</v>
-      </c>
-      <c r="CZ2">
-        <v>5.4492048120569403E-2</v>
-      </c>
-      <c r="DA2">
-        <v>5.7163876166543497E-2</v>
-      </c>
-      <c r="DB2">
-        <v>5.7794023766536501E-2</v>
-      </c>
-      <c r="DC2">
-        <v>6.0133236795870397E-2</v>
-      </c>
-      <c r="DD2">
-        <v>6.2280536463687697E-2</v>
-      </c>
-      <c r="DE2">
-        <v>6.3011917032779405E-2</v>
-      </c>
-      <c r="DF2">
-        <v>6.4032609217466799E-2</v>
-      </c>
-      <c r="DG2">
-        <v>6.4140414210958202E-2</v>
-      </c>
-      <c r="DH2">
-        <v>6.4338495280504407E-2</v>
-      </c>
-      <c r="DI2">
-        <v>6.3391732543089094E-2</v>
-      </c>
-      <c r="DJ2">
-        <v>6.2559625240011602E-2</v>
-      </c>
-      <c r="DK2">
-        <v>7.0344326693030201E-2</v>
-      </c>
-      <c r="DL2">
-        <v>7.7210379406574603E-2</v>
-      </c>
-      <c r="DM2">
-        <v>7.5506396387771901E-2</v>
-      </c>
-      <c r="DN2">
-        <v>7.3343915488567807E-2</v>
-      </c>
-      <c r="DO2">
-        <v>7.1323298214378106E-2</v>
-      </c>
-      <c r="DP2">
-        <v>7.1541853485627499E-2</v>
-      </c>
-      <c r="DQ2">
-        <v>7.1070268823942795E-2</v>
-      </c>
-      <c r="DR2">
-        <v>7.59616670872474E-2</v>
-      </c>
-      <c r="DS2">
-        <v>7.9025170775369802E-2</v>
-      </c>
-      <c r="DT2">
-        <v>8.3497008795980293E-2</v>
-      </c>
-      <c r="DU2">
-        <v>8.8495454333670898E-2</v>
-      </c>
-      <c r="DV2">
-        <v>9.3985194819147397E-2</v>
-      </c>
-      <c r="DW2">
-        <v>9.6608466626067105E-2</v>
-      </c>
-      <c r="DX2">
-        <v>9.44086928971275E-2</v>
-      </c>
-      <c r="DY2">
-        <v>9.58297433120395E-2</v>
-      </c>
-      <c r="DZ2">
-        <v>9.9149509147190895E-2</v>
-      </c>
-      <c r="EA2">
-        <v>0.10240207183137801</v>
-      </c>
-      <c r="EB2">
-        <v>8.8080562394497894E-2</v>
-      </c>
-      <c r="EC2">
-        <v>8.9800112061868803E-2</v>
-      </c>
-      <c r="ED2">
-        <v>8.9940473978330701E-2</v>
-      </c>
-      <c r="EE2">
-        <v>8.9420671883272199E-2</v>
-      </c>
-      <c r="EF2">
-        <v>8.9101524442151095E-2</v>
-      </c>
-      <c r="EG2">
-        <v>8.7990059332400797E-2</v>
-      </c>
-      <c r="EH2">
-        <v>8.7830697673587393E-2</v>
-      </c>
-      <c r="EI2">
-        <v>8.8729150997564801E-2</v>
-      </c>
-      <c r="EJ2">
-        <v>8.7730087414363805E-2</v>
-      </c>
-      <c r="EK2">
-        <v>8.8546035104806298E-2</v>
-      </c>
-      <c r="EL2">
-        <v>8.7561532454690699E-2</v>
-      </c>
-      <c r="EM2">
-        <v>8.6309175292286197E-2</v>
-      </c>
-      <c r="EN2">
-        <v>8.5133811599823001E-2</v>
-      </c>
-      <c r="EO2">
-        <v>8.3401451454898606E-2</v>
-      </c>
-      <c r="EP2">
-        <v>8.7369547639582101E-2</v>
-      </c>
-      <c r="EQ2">
-        <v>8.4658460990283999E-2</v>
-      </c>
-      <c r="ER2">
-        <v>9.5252573809335397E-2</v>
-      </c>
-      <c r="ES2">
-        <v>9.0965374569034502E-2</v>
-      </c>
-      <c r="ET2">
-        <v>8.6903040782383006E-2</v>
-      </c>
-      <c r="EU2">
-        <v>8.3658842557811003E-2</v>
-      </c>
-      <c r="EV2">
-        <v>8.0381743492809798E-2</v>
-      </c>
-      <c r="EW2">
-        <v>7.6855164318460706E-2</v>
-      </c>
-      <c r="EX2">
-        <v>7.5886630406427694E-2</v>
-      </c>
-      <c r="EY2">
-        <v>7.3323233566680801E-2</v>
-      </c>
-      <c r="EZ2">
-        <v>7.03346895105222E-2</v>
-      </c>
-      <c r="FA2">
-        <v>6.7194099421957199E-2</v>
-      </c>
-      <c r="FB2">
-        <v>6.5142649042183601E-2</v>
-      </c>
-      <c r="FC2">
-        <v>7.6672836712344997E-2</v>
-      </c>
-      <c r="FD2">
-        <v>7.4242298470049303E-2</v>
-      </c>
-      <c r="FE2">
-        <v>7.2602394551530905E-2</v>
-      </c>
-      <c r="FF2">
-        <v>7.3506133729747195E-2</v>
-      </c>
-      <c r="FG2">
-        <v>7.3082956776979194E-2</v>
-      </c>
-      <c r="FH2">
-        <v>7.1261369906972696E-2</v>
-      </c>
-      <c r="FI2">
-        <v>7.5673647722332996E-2</v>
-      </c>
-      <c r="FJ2">
-        <v>7.2862296939930501E-2</v>
-      </c>
-      <c r="FK2">
-        <v>7.6958818951244998E-2</v>
-      </c>
-      <c r="FL2">
-        <v>8.1544619025140805E-2</v>
-      </c>
-      <c r="FM2">
-        <v>7.1458857601879006E-2</v>
-      </c>
-      <c r="FN2">
-        <v>7.6924595223422196E-2</v>
-      </c>
-      <c r="FO2">
-        <v>8.1997290414881893E-2</v>
-      </c>
-      <c r="FP2">
-        <v>8.4574917944426703E-2</v>
-      </c>
-      <c r="FQ2">
-        <v>8.5626315439430098E-2</v>
-      </c>
-      <c r="FR2">
-        <v>8.6774440920707505E-2</v>
-      </c>
-      <c r="FS2">
-        <v>8.7496327126603601E-2</v>
-      </c>
-      <c r="FT2">
-        <v>8.7851185743623897E-2</v>
-      </c>
-      <c r="FU2">
-        <v>8.6596537458988695E-2</v>
-      </c>
-      <c r="FV2">
-        <v>8.4225670712307493E-2</v>
-      </c>
-      <c r="FW2">
-        <v>9.2752045565452801E-2</v>
-      </c>
-      <c r="FX2">
-        <v>9.4077888063453102E-2</v>
-      </c>
-      <c r="FY2">
-        <v>9.0493375641976195E-2</v>
-      </c>
-      <c r="FZ2">
-        <v>8.6472175966865503E-2</v>
-      </c>
-      <c r="GA2">
-        <v>8.3024907576413107E-2</v>
-      </c>
-      <c r="GB2">
-        <v>9.3677130612539294E-2</v>
-      </c>
-      <c r="GC2">
-        <v>9.6155648550436498E-2</v>
-      </c>
-      <c r="GD2">
-        <v>9.1979209761255704E-2</v>
-      </c>
-      <c r="GE2">
-        <v>0.11006901167984599</v>
-      </c>
-      <c r="GF2">
-        <v>0.10284983555117599</v>
-      </c>
-      <c r="GG2">
-        <v>9.6627557037829201E-2</v>
-      </c>
-      <c r="GH2">
-        <v>9.88076268442169E-2</v>
-      </c>
-      <c r="GI2">
-        <v>9.6435558936374705E-2</v>
-      </c>
-      <c r="GJ2">
-        <v>9.7091562832332307E-2</v>
-      </c>
-      <c r="GK2">
-        <v>6.2246957480945303E-2</v>
-      </c>
-      <c r="GL2">
-        <v>5.0601944065161102E-2</v>
-      </c>
-      <c r="GM2">
-        <v>5.7695114836403799E-2</v>
-      </c>
-      <c r="GN2">
-        <v>6.5231957690377304E-2</v>
-      </c>
-      <c r="GO2">
-        <v>7.3885503944917399E-2</v>
-      </c>
-      <c r="GP2">
-        <v>5.44867010278101E-2</v>
-      </c>
-      <c r="GQ2">
-        <v>6.0151474854133302E-2</v>
-      </c>
-      <c r="GR2">
-        <v>5.4588284980985301E-2</v>
-      </c>
-      <c r="GS2">
-        <v>5.9867829495097002E-2</v>
-      </c>
-      <c r="GT2">
-        <v>6.6490814187487202E-2</v>
-      </c>
-      <c r="GU2">
-        <v>7.3423837857614804E-2</v>
-      </c>
-      <c r="GV2">
-        <v>7.2399279258235805E-2</v>
-      </c>
-      <c r="GW2">
-        <v>7.8072519228778003E-2</v>
-      </c>
-      <c r="GX2">
-        <v>8.4315549187248595E-2</v>
-      </c>
-      <c r="GY2">
-        <v>7.4634009792752407E-2</v>
-      </c>
-      <c r="GZ2">
-        <v>7.4184361965681803E-2</v>
-      </c>
-      <c r="HA2">
-        <v>8.1387730818578502E-2</v>
-      </c>
-      <c r="HB2">
-        <v>8.7723400626332604E-2</v>
-      </c>
-      <c r="HC2">
-        <v>8.4390155995239302E-2</v>
-      </c>
-      <c r="HD2">
-        <v>8.9522727737690003E-2</v>
-      </c>
-      <c r="HE2">
-        <v>9.3983192786837699E-2</v>
-      </c>
-      <c r="HF2">
-        <v>9.0300439124021997E-2</v>
-      </c>
-      <c r="HG2">
-        <v>9.4686402263195399E-2</v>
-      </c>
-      <c r="HH2">
-        <v>9.6130812593367906E-2</v>
-      </c>
-      <c r="HI2">
-        <v>9.2980985203893196E-2</v>
-      </c>
-      <c r="HJ2">
-        <v>9.1886663893155807E-2</v>
-      </c>
-      <c r="HK2">
-        <v>9.3112630941761199E-2</v>
-      </c>
-      <c r="HL2">
-        <v>9.2331557932939304E-2</v>
-      </c>
-      <c r="HM2">
-        <v>9.37812086014021E-2</v>
-      </c>
-      <c r="HN2">
-        <v>9.5878411042679995E-2</v>
-      </c>
-      <c r="HO2">
-        <v>9.8477896299678097E-2</v>
-      </c>
-      <c r="HP2">
-        <v>9.6727519228440403E-2</v>
-      </c>
-      <c r="HQ2">
-        <v>9.6878387536869406E-2</v>
-      </c>
-      <c r="HR2">
-        <v>9.8766920244862597E-2</v>
-      </c>
-      <c r="HS2">
-        <v>9.4731056626623095E-2</v>
-      </c>
-      <c r="HT2">
-        <v>9.5673121208416007E-2</v>
-      </c>
-      <c r="HU2">
-        <v>9.4908968474161901E-2</v>
-      </c>
-      <c r="HV2">
-        <v>9.3381705881011898E-2</v>
-      </c>
-      <c r="HW2">
-        <v>9.3361250405555304E-2</v>
-      </c>
-      <c r="HX2">
-        <v>9.6388910800607797E-2</v>
-      </c>
-      <c r="HY2">
-        <v>9.5411261399929198E-2</v>
-      </c>
-      <c r="HZ2">
-        <v>9.4441788201127599E-2</v>
-      </c>
-      <c r="IA2">
-        <v>9.2484889966943901E-2</v>
-      </c>
-      <c r="IB2">
-        <v>8.9557261790498402E-2</v>
-      </c>
-      <c r="IC2">
-        <v>8.5489723394614997E-2</v>
-      </c>
-      <c r="ID2">
-        <v>8.70605480624419E-2</v>
-      </c>
-      <c r="IE2">
-        <v>2.5759320650292E-2</v>
-      </c>
-      <c r="IF2">
-        <v>2.8788306160243499E-2</v>
-      </c>
-      <c r="IG2">
-        <v>3.1795604385897798E-2</v>
-      </c>
-      <c r="IH2">
-        <v>3.4564735093059497E-2</v>
-      </c>
-      <c r="II2">
-        <v>3.68102971298543E-2</v>
-      </c>
-      <c r="IJ2">
-        <v>3.8849332085413003E-2</v>
-      </c>
-      <c r="IK2">
-        <v>4.0152134785636097E-2</v>
-      </c>
-      <c r="IL2">
-        <v>4.1883469604202202E-2</v>
-      </c>
-      <c r="IM2">
-        <v>4.5489165407062798E-2</v>
-      </c>
-      <c r="IN2">
-        <v>4.71675568587029E-2</v>
-      </c>
-      <c r="IO2">
-        <v>4.8708951612338298E-2</v>
-      </c>
-      <c r="IP2">
-        <v>5.0085398424166101E-2</v>
-      </c>
-      <c r="IQ2">
-        <v>5.2802011604845003E-2</v>
-      </c>
-      <c r="IR2">
-        <v>6.0620034232809601E-2</v>
-      </c>
-      <c r="IS2">
-        <v>6.2326903323394002E-2</v>
-      </c>
-      <c r="IT2">
-        <v>6.2334582086227303E-2</v>
-      </c>
-      <c r="IU2">
-        <v>6.2397748718477801E-2</v>
-      </c>
-      <c r="IV2">
-        <v>6.5735901284672701E-2</v>
-      </c>
-      <c r="IW2">
-        <v>6.4936687623017603E-2</v>
-      </c>
-      <c r="IX2">
-        <v>6.5484195495869799E-2</v>
-      </c>
-      <c r="IY2">
-        <v>6.7606921952117704E-2</v>
-      </c>
-      <c r="IZ2">
-        <v>6.6408082663590495E-2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:260" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>8.0412262509569496E-2</v>
-      </c>
-      <c r="B3">
-        <v>6.8114383081789895E-2</v>
-      </c>
-      <c r="C3">
-        <v>6.9459038718510793E-2</v>
-      </c>
-      <c r="D3">
-        <v>7.78581461950522E-2</v>
-      </c>
-      <c r="E3">
-        <v>7.34921022870825E-2</v>
-      </c>
-      <c r="F3">
-        <v>7.4378050213133304E-2</v>
-      </c>
-      <c r="G3">
-        <v>7.4691016129387597E-2</v>
-      </c>
-      <c r="H3">
-        <v>7.5172125892579794E-2</v>
-      </c>
-      <c r="I3">
-        <v>7.2076745494845301E-2</v>
-      </c>
-      <c r="J3">
-        <v>7.6273770812274502E-2</v>
-      </c>
-      <c r="K3">
-        <v>7.8323553558387701E-2</v>
-      </c>
-      <c r="L3">
-        <v>7.8900049193404598E-2</v>
-      </c>
-      <c r="M3">
-        <v>7.8740082018634902E-2</v>
-      </c>
-      <c r="N3">
-        <v>8.2520688893575597E-2</v>
-      </c>
-      <c r="O3">
-        <v>8.9308777644000997E-2</v>
-      </c>
-      <c r="P3">
-        <v>9.3371696766626697E-2</v>
-      </c>
-      <c r="Q3">
-        <v>9.6017016578975406E-2</v>
-      </c>
-      <c r="R3">
-        <v>7.7508499310819504E-2</v>
-      </c>
-      <c r="S3">
-        <v>9.0060037751781494E-2</v>
-      </c>
-      <c r="T3">
-        <v>9.7582307596855794E-2</v>
-      </c>
-      <c r="U3">
-        <v>0.110397607482437</v>
-      </c>
-      <c r="V3">
-        <v>6.4915497262227298E-2</v>
-      </c>
-      <c r="W3">
-        <v>5.0368442055243601E-2</v>
-      </c>
-      <c r="X3">
-        <v>5.5486372067909497E-2</v>
-      </c>
-      <c r="Y3">
-        <v>4.6033907819652602E-2</v>
-      </c>
-      <c r="Z3">
-        <v>5.4498548770953198E-2</v>
-      </c>
-      <c r="AA3">
-        <v>4.7802755981495901E-2</v>
-      </c>
-      <c r="AB3">
-        <v>4.4222075728205301E-2</v>
-      </c>
-      <c r="AC3">
-        <v>4.0980151773218697E-2</v>
-      </c>
-      <c r="AD3">
-        <v>3.81493771553389E-2</v>
-      </c>
-      <c r="AE3">
-        <v>3.7084277364334201E-2</v>
-      </c>
-      <c r="AF3">
-        <v>3.7423732058210001E-2</v>
-      </c>
-      <c r="AG3">
-        <v>3.6051175780210297E-2</v>
-      </c>
-      <c r="AH3">
-        <v>3.8991362706342E-2</v>
-      </c>
-      <c r="AI3">
-        <v>3.74877079570985E-2</v>
-      </c>
-      <c r="AJ3">
-        <v>4.0225874742104303E-2</v>
-      </c>
-      <c r="AK3">
-        <v>4.0791874340543301E-2</v>
-      </c>
-      <c r="AL3">
-        <v>4.3077264989655299E-2</v>
-      </c>
-      <c r="AM3">
-        <v>4.5970418815589102E-2</v>
-      </c>
-      <c r="AN3">
-        <v>4.8287914496835803E-2</v>
-      </c>
-      <c r="AO3">
-        <v>5.4558549491482901E-2</v>
-      </c>
-      <c r="AP3">
-        <v>5.6277459228902399E-2</v>
-      </c>
-      <c r="AQ3">
-        <v>5.6156177761322701E-2</v>
-      </c>
-      <c r="AR3">
-        <v>5.5714097629774799E-2</v>
-      </c>
-      <c r="AS3">
-        <v>5.6246392171006097E-2</v>
-      </c>
-      <c r="AT3">
-        <v>5.8310387983819101E-2</v>
-      </c>
-      <c r="AU3">
-        <v>6.0748706859581503E-2</v>
-      </c>
-      <c r="AV3">
-        <v>5.9565782419017901E-2</v>
-      </c>
-      <c r="AW3">
-        <v>6.9925104615074604E-2</v>
-      </c>
-      <c r="AX3">
-        <v>6.0152925478205402E-2</v>
-      </c>
-      <c r="AY3">
-        <v>5.0361559896089501E-2</v>
-      </c>
-      <c r="AZ3">
-        <v>4.7067865656518403E-2</v>
-      </c>
-      <c r="BA3">
-        <v>4.3580236786069197E-2</v>
-      </c>
-      <c r="BB3">
-        <v>4.4213205152333603E-2</v>
-      </c>
-      <c r="BC3">
-        <v>4.5761960794565598E-2</v>
-      </c>
-      <c r="BD3">
-        <v>5.0296194179796597E-2</v>
-      </c>
-      <c r="BE3">
-        <v>5.7815141399471297E-2</v>
-      </c>
-      <c r="BF3">
-        <v>4.4679945940811698E-2</v>
-      </c>
-      <c r="BG3">
-        <v>3.8031089056621899E-2</v>
-      </c>
-      <c r="BH3">
-        <v>4.2552628025776897E-2</v>
-      </c>
-      <c r="BI3">
-        <v>5.1657229030141902E-2</v>
-      </c>
-      <c r="BJ3">
-        <v>5.1512773028261703E-2</v>
-      </c>
-      <c r="BK3">
-        <v>4.8230585686746402E-2</v>
-      </c>
-      <c r="BL3">
-        <v>5.4563381713072998E-2</v>
-      </c>
-      <c r="BM3">
-        <v>6.4062163203844599E-2</v>
-      </c>
-      <c r="BN3">
-        <v>7.41189094443956E-2</v>
-      </c>
-      <c r="BO3">
-        <v>7.2161995693432401E-2</v>
-      </c>
-      <c r="BP3">
-        <v>7.1692323203137398E-2</v>
-      </c>
-      <c r="BQ3">
-        <v>6.9382450627631001E-2</v>
-      </c>
-      <c r="BR3">
-        <v>7.6452328360130301E-2</v>
-      </c>
-      <c r="BS3">
-        <v>6.7350983502477604E-2</v>
-      </c>
-      <c r="BT3">
-        <v>6.6995709412218496E-2</v>
-      </c>
-      <c r="BU3">
-        <v>5.9095264625725098E-2</v>
-      </c>
-      <c r="BV3">
-        <v>6.4281798672796903E-2</v>
-      </c>
-      <c r="BW3">
-        <v>6.2813931349028795E-2</v>
-      </c>
-      <c r="BX3">
-        <v>6.1520115924225099E-2</v>
-      </c>
-      <c r="BY3">
-        <v>6.19416199985654E-2</v>
-      </c>
-      <c r="BZ3">
-        <v>6.3422190947991994E-2</v>
-      </c>
-      <c r="CA3">
-        <v>7.0318173743967594E-2</v>
-      </c>
-      <c r="CB3">
-        <v>8.2470772684854601E-2</v>
-      </c>
-      <c r="CC3">
-        <v>9.6131894805018797E-2</v>
-      </c>
-      <c r="CD3">
-        <v>9.0539279815945603E-2</v>
-      </c>
-      <c r="CE3">
-        <v>7.9888892317827295E-2</v>
-      </c>
-      <c r="CF3">
-        <v>7.4357848846772295E-2</v>
-      </c>
-      <c r="CG3">
-        <v>6.2683913999372301E-2</v>
-      </c>
-      <c r="CH3">
-        <v>4.6098474388445297E-2</v>
-      </c>
-      <c r="CI3">
-        <v>3.8531441388039801E-2</v>
-      </c>
-      <c r="CJ3">
-        <v>5.0039602478243399E-2</v>
-      </c>
-      <c r="CK3">
-        <v>3.7288137380804401E-2</v>
-      </c>
-      <c r="CL3">
-        <v>3.4061759593704298E-2</v>
-      </c>
-      <c r="CM3">
-        <v>3.4424627797671498E-2</v>
-      </c>
-      <c r="CN3">
-        <v>4.0777271358494703E-2</v>
-      </c>
-      <c r="CO3">
-        <v>4.1319191553096497E-2</v>
-      </c>
-      <c r="CP3">
-        <v>4.0614418977424203E-2</v>
-      </c>
-      <c r="CQ3">
-        <v>4.41476804596415E-2</v>
-      </c>
-      <c r="CR3">
-        <v>4.5265781610698302E-2</v>
-      </c>
-      <c r="CS3">
-        <v>4.6166731207283297E-2</v>
-      </c>
-      <c r="CT3">
-        <v>4.9418414195628403E-2</v>
-      </c>
-      <c r="CU3">
-        <v>4.9758793340061398E-2</v>
-      </c>
-      <c r="CV3">
-        <v>5.1815555601508502E-2</v>
-      </c>
-      <c r="CW3">
-        <v>5.3254872439902103E-2</v>
-      </c>
-      <c r="CX3">
-        <v>5.5249764413682997E-2</v>
-      </c>
-      <c r="CY3">
-        <v>5.5858890401245503E-2</v>
-      </c>
-      <c r="CZ3">
-        <v>5.6546648205524699E-2</v>
-      </c>
-      <c r="DA3">
-        <v>5.9559138188203603E-2</v>
-      </c>
-      <c r="DB3">
-        <v>5.8746168215467E-2</v>
-      </c>
-      <c r="DC3">
-        <v>6.1423081494703401E-2</v>
-      </c>
-      <c r="DD3">
-        <v>6.2535059432468398E-2</v>
-      </c>
-      <c r="DE3">
-        <v>6.1960777616319102E-2</v>
-      </c>
-      <c r="DF3">
-        <v>6.4199450576394798E-2</v>
-      </c>
-      <c r="DG3">
-        <v>6.17871906376588E-2</v>
-      </c>
-      <c r="DH3">
-        <v>6.3757235346227001E-2</v>
-      </c>
-      <c r="DI3">
-        <v>6.7392852584853793E-2</v>
-      </c>
-      <c r="DJ3">
-        <v>7.2246001937914597E-2</v>
-      </c>
-      <c r="DK3">
-        <v>8.1202129069625095E-2</v>
-      </c>
-      <c r="DL3">
-        <v>9.2244345340760703E-2</v>
-      </c>
-      <c r="DM3">
-        <v>8.1006911253304101E-2</v>
-      </c>
-      <c r="DN3">
-        <v>7.2380137799712793E-2</v>
-      </c>
-      <c r="DO3">
-        <v>7.2403465304449299E-2</v>
-      </c>
-      <c r="DP3">
-        <v>7.6113677451424902E-2</v>
-      </c>
-      <c r="DQ3">
-        <v>7.1899506138129995E-2</v>
-      </c>
-      <c r="DR3">
-        <v>7.81870011390704E-2</v>
-      </c>
-      <c r="DS3">
-        <v>6.9449035661975606E-2</v>
-      </c>
-      <c r="DT3">
-        <v>7.9207798345135805E-2</v>
-      </c>
-      <c r="DU3">
-        <v>6.9320749709424506E-2</v>
-      </c>
-      <c r="DV3">
-        <v>6.8547838469994196E-2</v>
-      </c>
-      <c r="DW3">
-        <v>6.4888442715463707E-2</v>
-      </c>
-      <c r="DX3">
-        <v>6.1823531305803099E-2</v>
-      </c>
-      <c r="DY3">
-        <v>6.5537184379655999E-2</v>
-      </c>
-      <c r="DZ3">
-        <v>6.5737222100815798E-2</v>
-      </c>
-      <c r="EA3">
-        <v>7.0327075983761603E-2</v>
-      </c>
-      <c r="EB3">
-        <v>6.4749912347114594E-2</v>
-      </c>
-      <c r="EC3">
-        <v>6.4507187335108795E-2</v>
-      </c>
-      <c r="ED3">
-        <v>6.3702400508463597E-2</v>
-      </c>
-      <c r="EE3">
-        <v>6.44993516301616E-2</v>
-      </c>
-      <c r="EF3">
-        <v>6.5462736271049995E-2</v>
-      </c>
-      <c r="EG3">
-        <v>6.71784224926089E-2</v>
-      </c>
-      <c r="EH3">
-        <v>6.8130840411374002E-2</v>
-      </c>
-      <c r="EI3">
-        <v>7.0409152727839097E-2</v>
-      </c>
-      <c r="EJ3">
-        <v>6.9730595013302199E-2</v>
-      </c>
-      <c r="EK3">
-        <v>7.1056410513446105E-2</v>
-      </c>
-      <c r="EL3">
-        <v>6.9966897996453295E-2</v>
-      </c>
-      <c r="EM3">
-        <v>6.8738188592488106E-2</v>
-      </c>
-      <c r="EN3">
-        <v>7.0836526380826798E-2</v>
-      </c>
-      <c r="EO3">
-        <v>6.8071339248765905E-2</v>
-      </c>
-      <c r="EP3">
-        <v>7.0512802848333306E-2</v>
-      </c>
-      <c r="EQ3">
-        <v>6.5245074017470595E-2</v>
-      </c>
-      <c r="ER3">
-        <v>7.25218160134143E-2</v>
-      </c>
-      <c r="ES3">
-        <v>7.25856463351255E-2</v>
-      </c>
-      <c r="ET3">
-        <v>7.5124706583984097E-2</v>
-      </c>
-      <c r="EU3">
-        <v>7.6029117301079502E-2</v>
-      </c>
-      <c r="EV3">
-        <v>7.2892446073740402E-2</v>
-      </c>
-      <c r="EW3">
-        <v>8.0520734380711501E-2</v>
-      </c>
-      <c r="EX3">
-        <v>9.1171353466160704E-2</v>
-      </c>
-      <c r="EY3">
-        <v>7.8886875746069202E-2</v>
-      </c>
-      <c r="EZ3">
-        <v>8.0759447456570599E-2</v>
-      </c>
-      <c r="FA3">
-        <v>6.8460077115476706E-2</v>
-      </c>
-      <c r="FB3">
-        <v>6.8713521742040901E-2</v>
-      </c>
-      <c r="FC3">
-        <v>8.0000785161834606E-2</v>
-      </c>
-      <c r="FD3">
-        <v>7.0816769256526996E-2</v>
-      </c>
-      <c r="FE3">
-        <v>6.9150294353438002E-2</v>
-      </c>
-      <c r="FF3">
-        <v>6.9785759180693394E-2</v>
-      </c>
-      <c r="FG3">
-        <v>7.02818299550899E-2</v>
-      </c>
-      <c r="FH3">
-        <v>6.4492025974764597E-2</v>
-      </c>
-      <c r="FI3">
-        <v>7.1782294850801898E-2</v>
-      </c>
-      <c r="FJ3">
-        <v>6.4483224436535702E-2</v>
-      </c>
-      <c r="FK3">
-        <v>7.1224835693599595E-2</v>
-      </c>
-      <c r="FL3">
-        <v>7.1487544839950803E-2</v>
-      </c>
-      <c r="FM3">
-        <v>6.2878450106398795E-2</v>
-      </c>
-      <c r="FN3">
-        <v>6.1530280483732401E-2</v>
-      </c>
-      <c r="FO3">
-        <v>6.8408522165830501E-2</v>
-      </c>
-      <c r="FP3">
-        <v>7.2018909658204802E-2</v>
-      </c>
-      <c r="FQ3">
-        <v>7.2169558501021705E-2</v>
-      </c>
-      <c r="FR3">
-        <v>7.4843571809624296E-2</v>
-      </c>
-      <c r="FS3">
-        <v>7.5343245613807702E-2</v>
-      </c>
-      <c r="FT3">
-        <v>7.5876776504967602E-2</v>
-      </c>
-      <c r="FU3">
-        <v>7.4374607666311002E-2</v>
-      </c>
-      <c r="FV3">
-        <v>7.0410605348192407E-2</v>
-      </c>
-      <c r="FW3">
-        <v>7.3417207881463303E-2</v>
-      </c>
-      <c r="FX3">
-        <v>7.8907831934722297E-2</v>
-      </c>
-      <c r="FY3">
-        <v>7.4705734608150498E-2</v>
-      </c>
-      <c r="FZ3">
-        <v>8.0422864405055999E-2</v>
-      </c>
-      <c r="GA3">
-        <v>7.3692908007674598E-2</v>
-      </c>
-      <c r="GB3">
-        <v>7.6937953281358801E-2</v>
-      </c>
-      <c r="GC3">
-        <v>8.4411629672693694E-2</v>
-      </c>
-      <c r="GD3">
-        <v>7.8212733428918907E-2</v>
-      </c>
-      <c r="GE3">
-        <v>8.4897012824629997E-2</v>
-      </c>
-      <c r="GF3">
-        <v>7.9502777290545099E-2</v>
-      </c>
-      <c r="GG3">
-        <v>7.2732766886547298E-2</v>
-      </c>
-      <c r="GH3">
-        <v>7.5380057233865996E-2</v>
-      </c>
-      <c r="GI3">
-        <v>7.8229090884121305E-2</v>
-      </c>
-      <c r="GJ3">
-        <v>8.0723297079549505E-2</v>
-      </c>
-      <c r="GK3">
-        <v>6.8782529655361802E-2</v>
-      </c>
-      <c r="GL3">
-        <v>5.3541706547227799E-2</v>
-      </c>
-      <c r="GM3">
-        <v>6.7231428129439094E-2</v>
-      </c>
-      <c r="GN3">
-        <v>8.4736540816910802E-2</v>
-      </c>
-      <c r="GO3">
-        <v>0.112590255907631</v>
-      </c>
-      <c r="GP3">
-        <v>7.5320367989657702E-2</v>
-      </c>
-      <c r="GQ3">
-        <v>6.7426832834104902E-2</v>
-      </c>
-      <c r="GR3">
-        <v>5.7017893437401601E-2</v>
-      </c>
-      <c r="GS3">
-        <v>6.6861156060497695E-2</v>
-      </c>
-      <c r="GT3">
-        <v>8.7513394825962404E-2</v>
-      </c>
-      <c r="GU3">
-        <v>0.113642506195454</v>
-      </c>
-      <c r="GV3">
-        <v>7.8652832735388797E-2</v>
-      </c>
-      <c r="GW3">
-        <v>6.69832971412192E-2</v>
-      </c>
-      <c r="GX3">
-        <v>7.78413017874557E-2</v>
-      </c>
-      <c r="GY3">
-        <v>6.4796609021331594E-2</v>
-      </c>
-      <c r="GZ3">
-        <v>5.5320566168743202E-2</v>
-      </c>
-      <c r="HA3">
-        <v>6.5698649101143897E-2</v>
-      </c>
-      <c r="HB3">
-        <v>6.2252070429616703E-2</v>
-      </c>
-      <c r="HC3">
-        <v>5.4723601713159598E-2</v>
-      </c>
-      <c r="HD3">
-        <v>6.2754676097170101E-2</v>
-      </c>
-      <c r="HE3">
-        <v>6.7198171637221804E-2</v>
-      </c>
-      <c r="HF3">
-        <v>5.7181809087081599E-2</v>
-      </c>
-      <c r="HG3">
-        <v>6.6205512118146098E-2</v>
-      </c>
-      <c r="HH3">
-        <v>6.3486730595294499E-2</v>
-      </c>
-      <c r="HI3">
-        <v>5.9977834207037797E-2</v>
-      </c>
-      <c r="HJ3">
-        <v>5.8511167837382097E-2</v>
-      </c>
-      <c r="HK3">
-        <v>6.1866443032442001E-2</v>
-      </c>
-      <c r="HL3">
-        <v>6.0158343928544002E-2</v>
-      </c>
-      <c r="HM3">
-        <v>5.8660022885223199E-2</v>
-      </c>
-      <c r="HN3">
-        <v>6.3867286683798694E-2</v>
-      </c>
-      <c r="HO3">
-        <v>7.0928477531160106E-2</v>
-      </c>
-      <c r="HP3">
-        <v>6.6770246215576506E-2</v>
-      </c>
-      <c r="HQ3">
-        <v>6.4015257378480503E-2</v>
-      </c>
-      <c r="HR3">
-        <v>6.9640608149905303E-2</v>
-      </c>
-      <c r="HS3">
-        <v>6.6082654659158302E-2</v>
-      </c>
-      <c r="HT3">
-        <v>6.6127625445412105E-2</v>
-      </c>
-      <c r="HU3">
-        <v>6.7154841365048595E-2</v>
-      </c>
-      <c r="HV3">
-        <v>6.6843266537585697E-2</v>
-      </c>
-      <c r="HW3">
-        <v>6.93056553708115E-2</v>
-      </c>
-      <c r="HX3">
-        <v>7.2183225623216093E-2</v>
-      </c>
-      <c r="HY3">
-        <v>7.2538724396118998E-2</v>
-      </c>
-      <c r="HZ3">
-        <v>7.3736454013988095E-2</v>
-      </c>
-      <c r="IA3">
-        <v>7.4001922301065101E-2</v>
-      </c>
-      <c r="IB3">
-        <v>7.8143884829052296E-2</v>
-      </c>
-      <c r="IC3">
-        <v>8.14412137752904E-2</v>
-      </c>
-      <c r="ID3">
-        <v>8.4641994784528093E-2</v>
-      </c>
-      <c r="IE3">
-        <v>6.1989847642114501E-2</v>
-      </c>
-      <c r="IF3">
-        <v>6.9841849404114503E-2</v>
-      </c>
-      <c r="IG3">
-        <v>7.3541061105093897E-2</v>
-      </c>
-      <c r="IH3">
-        <v>7.65945241264816E-2</v>
-      </c>
-      <c r="II3">
-        <v>7.4585292821731403E-2</v>
-      </c>
-      <c r="IJ3">
-        <v>7.1211353000911901E-2</v>
-      </c>
-      <c r="IK3">
-        <v>6.2833048479952996E-2</v>
-      </c>
-      <c r="IL3">
-        <v>6.0675755749235803E-2</v>
-      </c>
-      <c r="IM3">
-        <v>6.4269537331031107E-2</v>
-      </c>
-      <c r="IN3">
-        <v>6.2794220107130705E-2</v>
-      </c>
-      <c r="IO3">
-        <v>6.4498869578919996E-2</v>
-      </c>
-      <c r="IP3">
-        <v>6.3145554608679405E-2</v>
-      </c>
-      <c r="IQ3">
-        <v>6.7833178949972706E-2</v>
-      </c>
-      <c r="IR3">
-        <v>7.3349325442376101E-2</v>
-      </c>
-      <c r="IS3">
-        <v>8.2442589183162093E-2</v>
-      </c>
-      <c r="IT3">
-        <v>7.6679777862155907E-2</v>
-      </c>
-      <c r="IU3">
-        <v>8.2429346065196599E-2</v>
-      </c>
-      <c r="IV3">
-        <v>9.2067968783158205E-2</v>
-      </c>
-      <c r="IW3">
-        <v>8.2008565393283606E-2</v>
-      </c>
-      <c r="IX3">
-        <v>7.8051148397214207E-2</v>
-      </c>
-      <c r="IY3">
-        <v>8.37248990583839E-2</v>
-      </c>
-      <c r="IZ3">
-        <v>7.6241930314511694E-2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:260" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>6.6995069777067595E-2</v>
-      </c>
-      <c r="B4">
-        <v>5.9383101983534997E-2</v>
-      </c>
-      <c r="C4">
-        <v>5.5052245780131397E-2</v>
-      </c>
-      <c r="D4">
-        <v>5.38982482817865E-2</v>
-      </c>
-      <c r="E4">
-        <v>5.3440617816242597E-2</v>
-      </c>
-      <c r="F4">
-        <v>5.4305174792082002E-2</v>
-      </c>
-      <c r="G4">
-        <v>5.4930500455099798E-2</v>
-      </c>
-      <c r="H4">
-        <v>5.5825090679014401E-2</v>
-      </c>
-      <c r="I4">
-        <v>5.5492148507642697E-2</v>
-      </c>
-      <c r="J4">
-        <v>5.6250263186023802E-2</v>
-      </c>
-      <c r="K4">
-        <v>5.6068468390209202E-2</v>
-      </c>
-      <c r="L4">
-        <v>5.7658158442343697E-2</v>
-      </c>
-      <c r="M4">
-        <v>5.8382491892244898E-2</v>
-      </c>
-      <c r="N4">
-        <v>6.0982409478506999E-2</v>
-      </c>
-      <c r="O4">
-        <v>6.3587232836654101E-2</v>
-      </c>
-      <c r="P4">
-        <v>6.7270801215682893E-2</v>
-      </c>
-      <c r="Q4">
-        <v>6.9141533836069594E-2</v>
-      </c>
-      <c r="R4">
-        <v>6.8209818059119701E-2</v>
-      </c>
-      <c r="S4">
-        <v>7.3798153433446201E-2</v>
-      </c>
-      <c r="T4">
-        <v>8.3553741389050196E-2</v>
-      </c>
-      <c r="U4">
-        <v>0.100491629353962</v>
-      </c>
-      <c r="V4">
-        <v>3.4045697193706398E-2</v>
-      </c>
-      <c r="W4">
-        <v>2.7426288902780701E-2</v>
-      </c>
-      <c r="X4">
-        <v>3.1370994087702497E-2</v>
-      </c>
-      <c r="Y4">
-        <v>3.3805616570239803E-2</v>
-      </c>
-      <c r="Z4">
-        <v>3.8254629206018798E-2</v>
-      </c>
-      <c r="AA4">
-        <v>4.0840198686045902E-2</v>
-      </c>
-      <c r="AB4">
-        <v>3.45349098321443E-2</v>
-      </c>
-      <c r="AC4">
-        <v>3.6104057268750198E-2</v>
-      </c>
-      <c r="AD4">
-        <v>3.1537513539868202E-2</v>
-      </c>
-      <c r="AE4">
-        <v>3.5609401970393299E-2</v>
-      </c>
-      <c r="AF4">
-        <v>4.0644827745274503E-2</v>
-      </c>
-      <c r="AG4">
-        <v>4.1702346210789699E-2</v>
-      </c>
-      <c r="AH4">
-        <v>4.6952152012803602E-2</v>
-      </c>
-      <c r="AI4">
-        <v>4.0652860530547903E-2</v>
-      </c>
-      <c r="AJ4">
-        <v>4.4792967832846899E-2</v>
-      </c>
-      <c r="AK4">
-        <v>4.6570913822641898E-2</v>
-      </c>
-      <c r="AL4">
-        <v>4.81816224190348E-2</v>
-      </c>
-      <c r="AM4">
-        <v>4.9439759542568802E-2</v>
-      </c>
-      <c r="AN4">
-        <v>5.00916247211406E-2</v>
-      </c>
-      <c r="AO4">
-        <v>6.2089591733109503E-2</v>
-      </c>
-      <c r="AP4">
-        <v>6.1577541717302599E-2</v>
-      </c>
-      <c r="AQ4">
-        <v>6.0589085808005101E-2</v>
-      </c>
-      <c r="AR4">
-        <v>5.9761025052178202E-2</v>
-      </c>
-      <c r="AS4">
-        <v>5.79675176656494E-2</v>
-      </c>
-      <c r="AT4">
-        <v>5.9768331419443599E-2</v>
-      </c>
-      <c r="AU4">
-        <v>6.2863090201846605E-2</v>
-      </c>
-      <c r="AV4">
-        <v>6.5972292640139596E-2</v>
-      </c>
-      <c r="AW4">
-        <v>7.1645511874048995E-2</v>
-      </c>
-      <c r="AX4">
-        <v>8.0892204740364196E-2</v>
-      </c>
-      <c r="AY4">
-        <v>4.5074322637864199E-2</v>
-      </c>
-      <c r="AZ4">
-        <v>3.8354695878006301E-2</v>
-      </c>
-      <c r="BA4">
-        <v>3.5957814420464203E-2</v>
-      </c>
-      <c r="BB4">
-        <v>3.5660123996270797E-2</v>
-      </c>
-      <c r="BC4">
-        <v>3.6707685995234003E-2</v>
-      </c>
-      <c r="BD4">
-        <v>4.1828054805465503E-2</v>
-      </c>
-      <c r="BE4">
-        <v>5.2005181997458898E-2</v>
-      </c>
-      <c r="BF4">
-        <v>4.7570774390710502E-2</v>
-      </c>
-      <c r="BG4">
-        <v>4.3438764271686602E-2</v>
-      </c>
-      <c r="BH4">
-        <v>4.1379514884589803E-2</v>
-      </c>
-      <c r="BI4">
-        <v>4.2506310048635101E-2</v>
-      </c>
-      <c r="BJ4">
-        <v>4.2106329574429502E-2</v>
-      </c>
-      <c r="BK4">
-        <v>4.2203755304713202E-2</v>
-      </c>
-      <c r="BL4">
-        <v>5.0748186337441298E-2</v>
-      </c>
-      <c r="BM4">
-        <v>5.1478035605734003E-2</v>
-      </c>
-      <c r="BN4">
-        <v>5.3188423845016097E-2</v>
-      </c>
-      <c r="BO4">
-        <v>5.3041235138825901E-2</v>
-      </c>
-      <c r="BP4">
-        <v>5.4064522133932598E-2</v>
-      </c>
-      <c r="BQ4">
-        <v>5.4090764840974699E-2</v>
-      </c>
-      <c r="BR4">
-        <v>5.5175527735737903E-2</v>
-      </c>
-      <c r="BS4">
-        <v>4.9898352131883601E-2</v>
-      </c>
-      <c r="BT4">
-        <v>5.3791734251976503E-2</v>
-      </c>
-      <c r="BU4">
-        <v>5.6631695577192699E-2</v>
-      </c>
-      <c r="BV4">
-        <v>5.9748887317752297E-2</v>
-      </c>
-      <c r="BW4">
-        <v>5.5114893500191602E-2</v>
-      </c>
-      <c r="BX4">
-        <v>5.6843348341571502E-2</v>
-      </c>
-      <c r="BY4">
-        <v>5.6205044886414E-2</v>
-      </c>
-      <c r="BZ4">
-        <v>5.7375549954828201E-2</v>
-      </c>
-      <c r="CA4">
-        <v>5.33687764652723E-2</v>
-      </c>
-      <c r="CB4">
-        <v>5.0060587368298902E-2</v>
-      </c>
-      <c r="CC4">
-        <v>5.7792178642157799E-2</v>
-      </c>
-      <c r="CD4">
-        <v>5.7292764080954697E-2</v>
-      </c>
-      <c r="CE4">
-        <v>5.4687429081918003E-2</v>
-      </c>
-      <c r="CF4">
-        <v>5.3306677244159897E-2</v>
-      </c>
-      <c r="CG4">
-        <v>4.9715519112385302E-2</v>
-      </c>
-      <c r="CH4">
-        <v>4.5012046693565698E-2</v>
-      </c>
-      <c r="CI4">
-        <v>4.1067983889803102E-2</v>
-      </c>
-      <c r="CJ4">
-        <v>4.8320857160178102E-2</v>
-      </c>
-      <c r="CK4">
-        <v>4.1794542191432298E-2</v>
-      </c>
-      <c r="CL4">
-        <v>3.7392429344441001E-2</v>
-      </c>
-      <c r="CM4">
-        <v>3.5248597551501601E-2</v>
-      </c>
-      <c r="CN4">
-        <v>4.7440867689193499E-2</v>
-      </c>
-      <c r="CO4">
-        <v>4.5272290568620303E-2</v>
-      </c>
-      <c r="CP4">
-        <v>4.4700169263701899E-2</v>
-      </c>
-      <c r="CQ4">
-        <v>4.5862112361122899E-2</v>
-      </c>
-      <c r="CR4">
-        <v>4.6295006838834502E-2</v>
-      </c>
-      <c r="CS4">
-        <v>4.6661869518262497E-2</v>
-      </c>
-      <c r="CT4">
-        <v>5.1162511042495501E-2</v>
-      </c>
-      <c r="CU4">
-        <v>5.1206256995581102E-2</v>
-      </c>
-      <c r="CV4">
-        <v>5.22458466087126E-2</v>
-      </c>
-      <c r="CW4">
-        <v>5.2993164751275801E-2</v>
-      </c>
-      <c r="CX4">
-        <v>5.4330317695726701E-2</v>
-      </c>
-      <c r="CY4">
-        <v>5.4518420185621003E-2</v>
-      </c>
-      <c r="CZ4">
-        <v>5.4884280925977101E-2</v>
-      </c>
-      <c r="DA4">
-        <v>5.4946262241070902E-2</v>
-      </c>
-      <c r="DB4">
-        <v>5.4753284636206601E-2</v>
-      </c>
-      <c r="DC4">
-        <v>5.74397708700101E-2</v>
-      </c>
-      <c r="DD4">
-        <v>5.7600045264809101E-2</v>
-      </c>
-      <c r="DE4">
-        <v>5.9104844938269903E-2</v>
-      </c>
-      <c r="DF4">
-        <v>6.0352763001317401E-2</v>
-      </c>
-      <c r="DG4">
-        <v>5.7032979716764499E-2</v>
-      </c>
-      <c r="DH4">
-        <v>5.9115586262394097E-2</v>
-      </c>
-      <c r="DI4">
-        <v>6.2211888372299802E-2</v>
-      </c>
-      <c r="DJ4">
-        <v>6.5950645950459894E-2</v>
-      </c>
-      <c r="DK4">
-        <v>6.9936408884607296E-2</v>
-      </c>
-      <c r="DL4">
-        <v>7.4207036445033306E-2</v>
-      </c>
-      <c r="DM4">
-        <v>7.3901752066990303E-2</v>
-      </c>
-      <c r="DN4">
-        <v>6.0542018656423502E-2</v>
-      </c>
-      <c r="DO4">
-        <v>6.3537478642594805E-2</v>
-      </c>
-      <c r="DP4">
-        <v>6.5263803656607694E-2</v>
-      </c>
-      <c r="DQ4">
-        <v>6.3519151794554807E-2</v>
-      </c>
-      <c r="DR4">
-        <v>6.0147609914841499E-2</v>
-      </c>
-      <c r="DS4">
-        <v>5.7273590158637797E-2</v>
-      </c>
-      <c r="DT4">
-        <v>5.5915077354956003E-2</v>
-      </c>
-      <c r="DU4">
-        <v>5.3090557389420201E-2</v>
-      </c>
-      <c r="DV4">
-        <v>5.1350768849352697E-2</v>
-      </c>
-      <c r="DW4">
-        <v>5.0659412157130101E-2</v>
-      </c>
-      <c r="DX4">
-        <v>5.0610732365365903E-2</v>
-      </c>
-      <c r="DY4">
-        <v>5.1444258158445597E-2</v>
-      </c>
-      <c r="DZ4">
-        <v>5.0757677630835198E-2</v>
-      </c>
-      <c r="EA4">
-        <v>5.0324827649696799E-2</v>
-      </c>
-      <c r="EB4">
-        <v>4.9702618007044397E-2</v>
-      </c>
-      <c r="EC4">
-        <v>4.9758289777202702E-2</v>
-      </c>
-      <c r="ED4">
-        <v>5.0247426906602902E-2</v>
-      </c>
-      <c r="EE4">
-        <v>5.1103747098816397E-2</v>
-      </c>
-      <c r="EF4">
-        <v>5.2145269642816301E-2</v>
-      </c>
-      <c r="EG4">
-        <v>5.3770883094527398E-2</v>
-      </c>
-      <c r="EH4">
-        <v>5.4719456158344497E-2</v>
-      </c>
-      <c r="EI4">
-        <v>5.5017883954930603E-2</v>
-      </c>
-      <c r="EJ4">
-        <v>5.5417344754917698E-2</v>
-      </c>
-      <c r="EK4">
-        <v>5.56103735213671E-2</v>
-      </c>
-      <c r="EL4">
-        <v>5.58498946477997E-2</v>
-      </c>
-      <c r="EM4">
-        <v>5.7203412076248301E-2</v>
-      </c>
-      <c r="EN4">
-        <v>5.8909759250011101E-2</v>
-      </c>
-      <c r="EO4">
-        <v>5.9797754309220401E-2</v>
-      </c>
-      <c r="EP4">
-        <v>6.1064349709746897E-2</v>
-      </c>
-      <c r="EQ4">
-        <v>5.9198795852612701E-2</v>
-      </c>
-      <c r="ER4">
-        <v>6.2108974036249598E-2</v>
-      </c>
-      <c r="ES4">
-        <v>6.5513833758270995E-2</v>
-      </c>
-      <c r="ET4">
-        <v>6.8861854642519801E-2</v>
-      </c>
-      <c r="EU4">
-        <v>7.1949471115278302E-2</v>
-      </c>
-      <c r="EV4">
-        <v>7.53403503505293E-2</v>
-      </c>
-      <c r="EW4">
-        <v>8.08454184436284E-2</v>
-      </c>
-      <c r="EX4">
-        <v>8.59788399250936E-2</v>
-      </c>
-      <c r="EY4">
-        <v>8.7299558209175801E-2</v>
-      </c>
-      <c r="EZ4">
-        <v>9.3775696975812298E-2</v>
-      </c>
-      <c r="FA4">
-        <v>8.9194465184427293E-2</v>
-      </c>
-      <c r="FB4">
-        <v>9.4495310789964801E-2</v>
-      </c>
-      <c r="FC4">
-        <v>0.104411834484557</v>
-      </c>
-      <c r="FD4">
-        <v>9.4791242128523398E-2</v>
-      </c>
-      <c r="FE4">
-        <v>9.8114216272922494E-2</v>
-      </c>
-      <c r="FF4">
-        <v>9.4678869281640099E-2</v>
-      </c>
-      <c r="FG4">
-        <v>9.1426610682942805E-2</v>
-      </c>
-      <c r="FH4">
-        <v>8.3653628590679194E-2</v>
-      </c>
-      <c r="FI4">
-        <v>0.10531290756320801</v>
-      </c>
-      <c r="FJ4">
-        <v>9.3185371263594302E-2</v>
-      </c>
-      <c r="FK4">
-        <v>0.11612370664732</v>
-      </c>
-      <c r="FL4">
-        <v>9.9987099388920406E-2</v>
-      </c>
-      <c r="FM4">
-        <v>8.61728278591741E-2</v>
-      </c>
-      <c r="FN4">
-        <v>7.6178513355876498E-2</v>
-      </c>
-      <c r="FO4">
-        <v>7.1502388734832098E-2</v>
-      </c>
-      <c r="FP4">
-        <v>6.9230848337348994E-2</v>
-      </c>
-      <c r="FQ4">
-        <v>6.8044169980476604E-2</v>
-      </c>
-      <c r="FR4">
-        <v>6.7488528071252593E-2</v>
-      </c>
-      <c r="FS4">
-        <v>6.6758371301447697E-2</v>
-      </c>
-      <c r="FT4">
-        <v>6.6863516483176802E-2</v>
-      </c>
-      <c r="FU4">
-        <v>6.3866831677318298E-2</v>
-      </c>
-      <c r="FV4">
-        <v>6.0029369184474601E-2</v>
-      </c>
-      <c r="FW4">
-        <v>6.18775079000616E-2</v>
-      </c>
-      <c r="FX4">
-        <v>6.39766806966722E-2</v>
-      </c>
-      <c r="FY4">
-        <v>5.8160251226447503E-2</v>
-      </c>
-      <c r="FZ4">
-        <v>6.18562612847132E-2</v>
-      </c>
-      <c r="GA4">
-        <v>5.4140629199297803E-2</v>
-      </c>
-      <c r="GB4">
-        <v>5.6468059101163898E-2</v>
-      </c>
-      <c r="GC4">
-        <v>5.9318541397087601E-2</v>
-      </c>
-      <c r="GD4">
-        <v>5.36775297734325E-2</v>
-      </c>
-      <c r="GE4">
-        <v>5.6371475735520801E-2</v>
-      </c>
-      <c r="GF4">
-        <v>5.8975076629246601E-2</v>
-      </c>
-      <c r="GG4">
-        <v>5.2631296067113503E-2</v>
-      </c>
-      <c r="GH4">
-        <v>5.4196723857296299E-2</v>
-      </c>
-      <c r="GI4">
-        <v>5.5919992494332202E-2</v>
-      </c>
-      <c r="GJ4">
-        <v>5.6290785278771502E-2</v>
-      </c>
-      <c r="GK4">
-        <v>5.2320500975223602E-2</v>
-      </c>
-      <c r="GL4">
-        <v>4.7262307445240202E-2</v>
-      </c>
-      <c r="GM4">
-        <v>7.3983658377475503E-2</v>
-      </c>
-      <c r="GN4">
-        <v>6.2447259160555699E-2</v>
-      </c>
-      <c r="GO4">
-        <v>9.7628222579004303E-2</v>
-      </c>
-      <c r="GP4">
-        <v>7.7363641049164794E-2</v>
-      </c>
-      <c r="GQ4">
-        <v>6.4693954031650402E-2</v>
-      </c>
-      <c r="GR4">
-        <v>5.8781051844230298E-2</v>
-      </c>
-      <c r="GS4">
-        <v>6.5828914058748203E-2</v>
-      </c>
-      <c r="GT4">
-        <v>6.5335578666708694E-2</v>
-      </c>
-      <c r="GU4">
-        <v>7.8035365727512102E-2</v>
-      </c>
-      <c r="GV4">
-        <v>6.6662411402037297E-2</v>
-      </c>
-      <c r="GW4">
-        <v>6.0580344316473397E-2</v>
-      </c>
-      <c r="GX4">
-        <v>7.6531470354456996E-2</v>
-      </c>
-      <c r="GY4">
-        <v>6.9672150876045294E-2</v>
-      </c>
-      <c r="GZ4">
-        <v>6.2699166553278604E-2</v>
-      </c>
-      <c r="HA4">
-        <v>6.8974946339366905E-2</v>
-      </c>
-      <c r="HB4">
-        <v>6.2679717757086001E-2</v>
-      </c>
-      <c r="HC4">
-        <v>5.7510604685762003E-2</v>
-      </c>
-      <c r="HD4">
-        <v>5.7190685181975003E-2</v>
-      </c>
-      <c r="HE4">
-        <v>5.4268000614563099E-2</v>
-      </c>
-      <c r="HF4">
-        <v>5.1578330300977797E-2</v>
-      </c>
-      <c r="HG4">
-        <v>5.2674362324404499E-2</v>
-      </c>
-      <c r="HH4">
-        <v>5.2006722275782603E-2</v>
-      </c>
-      <c r="HI4">
-        <v>5.1624948976845997E-2</v>
-      </c>
-      <c r="HJ4">
-        <v>5.1767427964415198E-2</v>
-      </c>
-      <c r="HK4">
-        <v>5.60785298596123E-2</v>
-      </c>
-      <c r="HL4">
-        <v>5.5795890990211802E-2</v>
-      </c>
-      <c r="HM4">
-        <v>5.4872882923649398E-2</v>
-      </c>
-      <c r="HN4">
-        <v>5.9117786460897902E-2</v>
-      </c>
-      <c r="HO4">
-        <v>5.9716167921888101E-2</v>
-      </c>
-      <c r="HP4">
-        <v>5.85954242410422E-2</v>
-      </c>
-      <c r="HQ4">
-        <v>5.7644256693045598E-2</v>
-      </c>
-      <c r="HR4">
-        <v>5.78916053560369E-2</v>
-      </c>
-      <c r="HS4">
-        <v>5.7165868230251403E-2</v>
-      </c>
-      <c r="HT4">
-        <v>5.6704732346240801E-2</v>
-      </c>
-      <c r="HU4">
-        <v>5.7449870658622899E-2</v>
-      </c>
-      <c r="HV4">
-        <v>5.6774670062228999E-2</v>
-      </c>
-      <c r="HW4">
-        <v>5.79960509179792E-2</v>
-      </c>
-      <c r="HX4">
-        <v>5.9338917508863998E-2</v>
-      </c>
-      <c r="HY4">
-        <v>5.9669728465723798E-2</v>
-      </c>
-      <c r="HZ4">
-        <v>6.0478868239432597E-2</v>
-      </c>
-      <c r="IA4">
-        <v>6.1941215013092098E-2</v>
-      </c>
-      <c r="IB4">
-        <v>6.4615945987091999E-2</v>
-      </c>
-      <c r="IC4">
-        <v>6.7738069637886894E-2</v>
-      </c>
-      <c r="ID4">
-        <v>6.6858937849569602E-2</v>
-      </c>
-      <c r="IE4">
-        <v>4.9464089255749799E-2</v>
-      </c>
-      <c r="IF4">
-        <v>6.1382644599150098E-2</v>
-      </c>
-      <c r="IG4">
-        <v>5.89481240892984E-2</v>
-      </c>
-      <c r="IH4">
-        <v>6.3820946637806006E-2</v>
-      </c>
-      <c r="II4">
-        <v>5.9909522106386497E-2</v>
-      </c>
-      <c r="IJ4">
-        <v>5.6076226347152397E-2</v>
-      </c>
-      <c r="IK4">
-        <v>5.1125606073112097E-2</v>
-      </c>
-      <c r="IL4">
-        <v>4.6887550977966701E-2</v>
-      </c>
-      <c r="IM4">
-        <v>4.9077492573730702E-2</v>
-      </c>
-      <c r="IN4">
-        <v>4.6919776796243998E-2</v>
-      </c>
-      <c r="IO4">
-        <v>4.9297560202466201E-2</v>
-      </c>
-      <c r="IP4">
-        <v>5.1529436095545701E-2</v>
-      </c>
-      <c r="IQ4">
-        <v>5.3887267504804499E-2</v>
-      </c>
-      <c r="IR4">
-        <v>5.7003359885135003E-2</v>
-      </c>
-      <c r="IS4">
-        <v>6.0504264136058902E-2</v>
-      </c>
-      <c r="IT4">
-        <v>5.4037773265895997E-2</v>
-      </c>
-      <c r="IU4">
-        <v>5.7067998103141802E-2</v>
-      </c>
-      <c r="IV4">
-        <v>6.0485458313519397E-2</v>
-      </c>
-      <c r="IW4">
-        <v>6.2140414921322898E-2</v>
-      </c>
-      <c r="IX4">
-        <v>6.2187389883091103E-2</v>
-      </c>
-      <c r="IY4">
-        <v>6.44674364999855E-2</v>
-      </c>
-      <c r="IZ4">
-        <v>6.7016315196676196E-2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:260" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>6.8916963130112897E-3</v>
-      </c>
-      <c r="B5">
-        <v>6.6947777537752296E-3</v>
-      </c>
-      <c r="C5">
-        <v>6.5694239528873398E-3</v>
-      </c>
-      <c r="D5">
-        <v>6.5066556469104897E-3</v>
-      </c>
-      <c r="E5">
-        <v>6.4968667874356302E-3</v>
-      </c>
-      <c r="F5">
-        <v>6.5225950092097501E-3</v>
-      </c>
-      <c r="G5">
-        <v>6.5426726953727501E-3</v>
-      </c>
-      <c r="H5">
-        <v>6.5700215474277096E-3</v>
-      </c>
-      <c r="I5">
-        <v>6.5627057647427598E-3</v>
-      </c>
-      <c r="J5">
-        <v>6.5561326845388398E-3</v>
-      </c>
-      <c r="K5">
-        <v>6.5530386207786704E-3</v>
-      </c>
-      <c r="L5">
-        <v>6.6002263600015102E-3</v>
-      </c>
-      <c r="M5">
-        <v>6.6248256577846098E-3</v>
-      </c>
-      <c r="N5">
-        <v>6.6965525752535303E-3</v>
-      </c>
-      <c r="O5">
-        <v>6.7654419200132796E-3</v>
-      </c>
-      <c r="P5">
-        <v>6.8558470713087202E-3</v>
-      </c>
-      <c r="Q5">
-        <v>6.9014328750802599E-3</v>
-      </c>
-      <c r="R5">
-        <v>7.02567040634556E-3</v>
-      </c>
-      <c r="S5">
-        <v>7.1554512661601097E-3</v>
-      </c>
-      <c r="T5">
-        <v>7.3605468688944303E-3</v>
-      </c>
-      <c r="U5">
-        <v>7.6753437563969497E-3</v>
-      </c>
-      <c r="V5">
-        <v>3.3878969012888999E-3</v>
-      </c>
-      <c r="W5">
-        <v>3.2595629017259701E-3</v>
-      </c>
-      <c r="X5">
-        <v>3.38397702251246E-3</v>
-      </c>
-      <c r="Y5">
-        <v>3.5203662386050702E-3</v>
-      </c>
-      <c r="Z5">
-        <v>3.6649091419942402E-3</v>
-      </c>
-      <c r="AA5">
-        <v>3.8137665707370801E-3</v>
-      </c>
-      <c r="AB5">
-        <v>3.61762218469969E-3</v>
-      </c>
-      <c r="AC5">
-        <v>3.7601863980357602E-3</v>
-      </c>
-      <c r="AD5">
-        <v>3.8645771998949601E-3</v>
-      </c>
-      <c r="AE5">
-        <v>4.02658610305116E-3</v>
-      </c>
-      <c r="AF5">
-        <v>4.1951182529578598E-3</v>
-      </c>
-      <c r="AG5">
-        <v>4.3641382991944999E-3</v>
-      </c>
-      <c r="AH5">
-        <v>4.5443902296030099E-3</v>
-      </c>
-      <c r="AI5">
-        <v>4.6800476898814199E-3</v>
-      </c>
-      <c r="AJ5">
-        <v>4.8484236863751496E-3</v>
-      </c>
-      <c r="AK5">
-        <v>4.9913731998443402E-3</v>
-      </c>
-      <c r="AL5">
-        <v>5.1095167867456596E-3</v>
-      </c>
-      <c r="AM5">
-        <v>5.2068339353799099E-3</v>
-      </c>
-      <c r="AN5">
-        <v>5.3012366114810298E-3</v>
-      </c>
-      <c r="AO5">
-        <v>6.6163053660651403E-3</v>
-      </c>
-      <c r="AP5">
-        <v>6.6157376688616197E-3</v>
-      </c>
-      <c r="AQ5">
-        <v>6.60240553156857E-3</v>
-      </c>
-      <c r="AR5">
-        <v>6.5917042766932103E-3</v>
-      </c>
-      <c r="AS5">
-        <v>6.5548862086808402E-3</v>
-      </c>
-      <c r="AT5">
-        <v>6.7512600190665004E-3</v>
-      </c>
-      <c r="AU5">
-        <v>6.8289268791818201E-3</v>
-      </c>
-      <c r="AV5">
-        <v>6.9114204533514299E-3</v>
-      </c>
-      <c r="AW5">
-        <v>7.0423833708673899E-3</v>
-      </c>
-      <c r="AX5">
-        <v>7.2823979115947098E-3</v>
-      </c>
-      <c r="AY5">
-        <v>4.1085739292283704E-3</v>
-      </c>
-      <c r="AZ5">
-        <v>3.8496027979110698E-3</v>
-      </c>
-      <c r="BA5">
-        <v>3.9889976002494302E-3</v>
-      </c>
-      <c r="BB5">
-        <v>3.9896399024624404E-3</v>
-      </c>
-      <c r="BC5">
-        <v>4.0741069654731303E-3</v>
-      </c>
-      <c r="BD5">
-        <v>4.4397006912700104E-3</v>
-      </c>
-      <c r="BE5">
-        <v>4.84747507448765E-3</v>
-      </c>
-      <c r="BF5">
-        <v>4.8750801398462903E-3</v>
-      </c>
-      <c r="BG5">
-        <v>4.9005974395379698E-3</v>
-      </c>
-      <c r="BH5">
-        <v>4.9436325377063698E-3</v>
-      </c>
-      <c r="BI5">
-        <v>4.99556146900265E-3</v>
-      </c>
-      <c r="BJ5">
-        <v>5.0720097223669498E-3</v>
-      </c>
-      <c r="BK5">
-        <v>5.1433536379995497E-3</v>
-      </c>
-      <c r="BL5">
-        <v>5.3905966231776901E-3</v>
-      </c>
-      <c r="BM5">
-        <v>5.4278130961179904E-3</v>
-      </c>
-      <c r="BN5">
-        <v>5.47186998612504E-3</v>
-      </c>
-      <c r="BO5">
-        <v>5.5437210734401001E-3</v>
-      </c>
-      <c r="BP5">
-        <v>5.6387311145832597E-3</v>
-      </c>
-      <c r="BQ5">
-        <v>5.7035442762964602E-3</v>
-      </c>
-      <c r="BR5">
-        <v>5.7465364452699398E-3</v>
-      </c>
-      <c r="BS5">
-        <v>5.8438193295668097E-3</v>
-      </c>
-      <c r="BT5">
-        <v>5.9780810223228498E-3</v>
-      </c>
-      <c r="BU5">
-        <v>6.1291152706115801E-3</v>
-      </c>
-      <c r="BV5">
-        <v>6.2493912931263001E-3</v>
-      </c>
-      <c r="BW5">
-        <v>5.6982523781464603E-3</v>
-      </c>
-      <c r="BX5">
-        <v>5.8041137598672399E-3</v>
-      </c>
-      <c r="BY5">
-        <v>5.8680249048631604E-3</v>
-      </c>
-      <c r="BZ5">
-        <v>5.95748293297255E-3</v>
-      </c>
-      <c r="CA5">
-        <v>5.9238175615437703E-3</v>
-      </c>
-      <c r="CB5">
-        <v>5.8783244886145601E-3</v>
-      </c>
-      <c r="CC5">
-        <v>5.92098989299645E-3</v>
-      </c>
-      <c r="CD5">
-        <v>5.9665083816388097E-3</v>
-      </c>
-      <c r="CE5">
-        <v>5.9625926738349003E-3</v>
-      </c>
-      <c r="CF5">
-        <v>5.9776112015365902E-3</v>
-      </c>
-      <c r="CG5">
-        <v>5.9322643465869298E-3</v>
-      </c>
-      <c r="CH5">
-        <v>5.8222307894452603E-3</v>
-      </c>
-      <c r="CI5">
-        <v>5.7211906095809301E-3</v>
-      </c>
-      <c r="CJ5">
-        <v>5.6099111027540297E-3</v>
-      </c>
-      <c r="CK5">
-        <v>5.48557531298323E-3</v>
-      </c>
-      <c r="CL5">
-        <v>5.4032774332702796E-3</v>
-      </c>
-      <c r="CM5">
-        <v>5.3723610481731902E-3</v>
-      </c>
-      <c r="CN5">
-        <v>5.8812911797139298E-3</v>
-      </c>
-      <c r="CO5">
-        <v>5.8536008698783096E-3</v>
-      </c>
-      <c r="CP5">
-        <v>5.8660316263044604E-3</v>
-      </c>
-      <c r="CQ5">
-        <v>5.9058227228564698E-3</v>
-      </c>
-      <c r="CR5">
-        <v>5.9462055001702997E-3</v>
-      </c>
-      <c r="CS5">
-        <v>5.9822658705446499E-3</v>
-      </c>
-      <c r="CT5">
-        <v>6.5838542351717797E-3</v>
-      </c>
-      <c r="CU5">
-        <v>6.57244175333495E-3</v>
-      </c>
-      <c r="CV5">
-        <v>6.5924711382335296E-3</v>
-      </c>
-      <c r="CW5">
-        <v>6.60607526680032E-3</v>
-      </c>
-      <c r="CX5">
-        <v>6.6271335569997704E-3</v>
-      </c>
-      <c r="CY5">
-        <v>6.6243438117165303E-3</v>
-      </c>
-      <c r="CZ5">
-        <v>6.6280596111742704E-3</v>
-      </c>
-      <c r="DA5">
-        <v>6.6180999417636702E-3</v>
-      </c>
-      <c r="DB5">
-        <v>6.6060839998976599E-3</v>
-      </c>
-      <c r="DC5">
-        <v>6.6378114861880702E-3</v>
-      </c>
-      <c r="DD5">
-        <v>6.6414164788397602E-3</v>
-      </c>
-      <c r="DE5">
-        <v>6.6908009396044197E-3</v>
-      </c>
-      <c r="DF5">
-        <v>6.7251096470685098E-3</v>
-      </c>
-      <c r="DG5">
-        <v>6.7551011235133301E-3</v>
-      </c>
-      <c r="DH5">
-        <v>6.8056596741560898E-3</v>
-      </c>
-      <c r="DI5">
-        <v>6.8858451987859502E-3</v>
-      </c>
-      <c r="DJ5">
-        <v>6.9800583056178903E-3</v>
-      </c>
-      <c r="DK5">
-        <v>7.0749550743524096E-3</v>
-      </c>
-      <c r="DL5">
-        <v>7.1691164270506601E-3</v>
-      </c>
-      <c r="DM5">
-        <v>7.2286095671607502E-3</v>
-      </c>
-      <c r="DN5">
-        <v>7.0448381918799697E-3</v>
-      </c>
-      <c r="DO5">
-        <v>7.1080125639987803E-3</v>
-      </c>
-      <c r="DP5">
-        <v>7.1326868359638798E-3</v>
-      </c>
-      <c r="DQ5">
-        <v>7.0606213757404201E-3</v>
-      </c>
-      <c r="DR5">
-        <v>6.9321652231977698E-3</v>
-      </c>
-      <c r="DS5">
-        <v>6.8310578681641297E-3</v>
-      </c>
-      <c r="DT5">
-        <v>6.7347364024947501E-3</v>
-      </c>
-      <c r="DU5">
-        <v>6.6402608067294101E-3</v>
-      </c>
-      <c r="DV5">
-        <v>6.5812392906639096E-3</v>
-      </c>
-      <c r="DW5">
-        <v>6.5479752914298396E-3</v>
-      </c>
-      <c r="DX5">
-        <v>6.5315685751099004E-3</v>
-      </c>
-      <c r="DY5">
-        <v>6.5318662338613E-3</v>
-      </c>
-      <c r="DZ5">
-        <v>6.5101796456222003E-3</v>
-      </c>
-      <c r="EA5">
-        <v>6.4858570639964204E-3</v>
-      </c>
-      <c r="EB5">
-        <v>6.4560346966607302E-3</v>
-      </c>
-      <c r="EC5">
-        <v>6.4552128800539404E-3</v>
-      </c>
-      <c r="ED5">
-        <v>6.46505625420387E-3</v>
-      </c>
-      <c r="EE5">
-        <v>6.4986057698537799E-3</v>
-      </c>
-      <c r="EF5">
-        <v>6.5264428833745102E-3</v>
-      </c>
-      <c r="EG5">
-        <v>6.5708346795631898E-3</v>
-      </c>
-      <c r="EH5">
-        <v>6.5955948608045099E-3</v>
-      </c>
-      <c r="EI5">
-        <v>6.5985257773488798E-3</v>
-      </c>
-      <c r="EJ5">
-        <v>6.6067709828188104E-3</v>
-      </c>
-      <c r="EK5">
-        <v>6.6111997519228303E-3</v>
-      </c>
-      <c r="EL5">
-        <v>6.61497998410267E-3</v>
-      </c>
-      <c r="EM5">
-        <v>6.6592973758628398E-3</v>
-      </c>
-      <c r="EN5">
-        <v>6.7036152959391001E-3</v>
-      </c>
-      <c r="EO5">
-        <v>6.7536820592526301E-3</v>
-      </c>
-      <c r="EP5">
-        <v>6.7864067649577196E-3</v>
-      </c>
-      <c r="EQ5">
-        <v>6.8539653940708099E-3</v>
-      </c>
-      <c r="ER5">
-        <v>6.9331334168228802E-3</v>
-      </c>
-      <c r="ES5">
-        <v>7.0007595164819801E-3</v>
-      </c>
-      <c r="ET5">
-        <v>7.0659532877307904E-3</v>
-      </c>
-      <c r="EU5">
-        <v>7.1222698309908704E-3</v>
-      </c>
-      <c r="EV5">
-        <v>7.1909153674351396E-3</v>
-      </c>
-      <c r="EW5">
-        <v>7.29664546463492E-3</v>
-      </c>
-      <c r="EX5">
-        <v>7.3924671028587803E-3</v>
-      </c>
-      <c r="EY5">
-        <v>7.4685980682736202E-3</v>
-      </c>
-      <c r="EZ5">
-        <v>7.5643173785952802E-3</v>
-      </c>
-      <c r="FA5">
-        <v>7.7108459642696199E-3</v>
-      </c>
-      <c r="FB5">
-        <v>7.7870456348018199E-3</v>
-      </c>
-      <c r="FC5">
-        <v>7.9378180328899609E-3</v>
-      </c>
-      <c r="FD5">
-        <v>8.0046580816271404E-3</v>
-      </c>
-      <c r="FE5">
-        <v>8.0288845255704101E-3</v>
-      </c>
-      <c r="FF5">
-        <v>7.9299793338878394E-3</v>
-      </c>
-      <c r="FG5">
-        <v>7.8263949945210007E-3</v>
-      </c>
-      <c r="FH5">
-        <v>7.6320589006028203E-3</v>
-      </c>
-      <c r="FI5">
-        <v>8.1928450717959206E-3</v>
-      </c>
-      <c r="FJ5">
-        <v>7.9192214004272996E-3</v>
-      </c>
-      <c r="FK5">
-        <v>8.4745317726981993E-3</v>
-      </c>
-      <c r="FL5">
-        <v>8.1316963262731898E-3</v>
-      </c>
-      <c r="FM5">
-        <v>7.80785513217447E-3</v>
-      </c>
-      <c r="FN5">
-        <v>7.5401922309553298E-3</v>
-      </c>
-      <c r="FO5">
-        <v>7.3412429232699401E-3</v>
-      </c>
-      <c r="FP5">
-        <v>7.2429471371094302E-3</v>
-      </c>
-      <c r="FQ5">
-        <v>7.1915695563063197E-3</v>
-      </c>
-      <c r="FR5">
-        <v>7.1415175106323697E-3</v>
-      </c>
-      <c r="FS5">
-        <v>7.1051198602951303E-3</v>
-      </c>
-      <c r="FT5">
-        <v>7.0904855162907798E-3</v>
-      </c>
-      <c r="FU5">
-        <v>7.0165214157688503E-3</v>
-      </c>
-      <c r="FV5">
-        <v>7.0253018523493901E-3</v>
-      </c>
-      <c r="FW5">
-        <v>7.0570517385419498E-3</v>
-      </c>
-      <c r="FX5">
-        <v>7.0970926568076197E-3</v>
-      </c>
-      <c r="FY5">
-        <v>6.4942754447436298E-3</v>
-      </c>
-      <c r="FZ5">
-        <v>6.5988839751244602E-3</v>
-      </c>
-      <c r="GA5">
-        <v>6.4049956780651398E-3</v>
-      </c>
-      <c r="GB5">
-        <v>6.4802258212495302E-3</v>
-      </c>
-      <c r="GC5">
-        <v>6.5675147555739402E-3</v>
-      </c>
-      <c r="GD5">
-        <v>6.2894004704763598E-3</v>
-      </c>
-      <c r="GE5">
-        <v>6.37939484664477E-3</v>
-      </c>
-      <c r="GF5">
-        <v>6.4691239016216604E-3</v>
-      </c>
-      <c r="GG5">
-        <v>6.4194673602626503E-3</v>
-      </c>
-      <c r="GH5">
-        <v>6.47163383358148E-3</v>
-      </c>
-      <c r="GI5">
-        <v>6.5258876006490602E-3</v>
-      </c>
-      <c r="GJ5">
-        <v>6.5329805686459401E-3</v>
-      </c>
-      <c r="GK5">
-        <v>6.4270676794106396E-3</v>
-      </c>
-      <c r="GL5">
-        <v>6.2763638693070804E-3</v>
-      </c>
-      <c r="GM5">
-        <v>8.1415055031422209E-3</v>
-      </c>
-      <c r="GN5">
-        <v>7.60938406488004E-3</v>
-      </c>
-      <c r="GO5">
-        <v>8.0505724570653307E-3</v>
-      </c>
-      <c r="GP5">
-        <v>7.5786232613763403E-3</v>
-      </c>
-      <c r="GQ5">
-        <v>7.2639281117270098E-3</v>
-      </c>
-      <c r="GR5">
-        <v>7.0432357668316799E-3</v>
-      </c>
-      <c r="GS5">
-        <v>6.8695167217370304E-3</v>
-      </c>
-      <c r="GT5">
-        <v>6.6795451268817502E-3</v>
-      </c>
-      <c r="GU5">
-        <v>6.5578087468424404E-3</v>
-      </c>
-      <c r="GV5">
-        <v>6.4046566822221701E-3</v>
-      </c>
-      <c r="GW5">
-        <v>6.3083984714381799E-3</v>
-      </c>
-      <c r="GX5">
-        <v>6.4632069218761501E-3</v>
-      </c>
-      <c r="GY5">
-        <v>6.3703248682300201E-3</v>
-      </c>
-      <c r="GZ5">
-        <v>6.2794504294704902E-3</v>
-      </c>
-      <c r="HA5">
-        <v>6.19108798728035E-3</v>
-      </c>
-      <c r="HB5">
-        <v>6.1310373204186402E-3</v>
-      </c>
-      <c r="HC5">
-        <v>6.0747386750138197E-3</v>
-      </c>
-      <c r="HD5">
-        <v>6.0432392777578199E-3</v>
-      </c>
-      <c r="HE5">
-        <v>6.0314503427356496E-3</v>
-      </c>
-      <c r="HF5">
-        <v>5.9949401039264202E-3</v>
-      </c>
-      <c r="HG5">
-        <v>5.9901209258705701E-3</v>
-      </c>
-      <c r="HH5">
-        <v>6.0118269239058299E-3</v>
-      </c>
-      <c r="HI5">
-        <v>6.0322264563871303E-3</v>
-      </c>
-      <c r="HJ5">
-        <v>6.0649623061074902E-3</v>
-      </c>
-      <c r="HK5">
-        <v>6.2425754572881798E-3</v>
-      </c>
-      <c r="HL5">
-        <v>6.2580462536031703E-3</v>
-      </c>
-      <c r="HM5">
-        <v>6.2588737535790003E-3</v>
-      </c>
-      <c r="HN5">
-        <v>6.2810295374687202E-3</v>
-      </c>
-      <c r="HO5">
-        <v>6.2734041968153598E-3</v>
-      </c>
-      <c r="HP5">
-        <v>6.2755548785450701E-3</v>
-      </c>
-      <c r="HQ5">
-        <v>6.2797873803735098E-3</v>
-      </c>
-      <c r="HR5">
-        <v>6.28310369124741E-3</v>
-      </c>
-      <c r="HS5">
-        <v>6.2893732773660104E-3</v>
-      </c>
-      <c r="HT5">
-        <v>6.3071404813470197E-3</v>
-      </c>
-      <c r="HU5">
-        <v>6.3499017835324896E-3</v>
-      </c>
-      <c r="HV5">
-        <v>6.3869391844239903E-3</v>
-      </c>
-      <c r="HW5">
-        <v>6.4384321493038202E-3</v>
-      </c>
-      <c r="HX5">
-        <v>6.4916113430644601E-3</v>
-      </c>
-      <c r="HY5">
-        <v>6.5218293459596401E-3</v>
-      </c>
-      <c r="HZ5">
-        <v>6.5565143179210101E-3</v>
-      </c>
-      <c r="IA5">
-        <v>6.6034310897541198E-3</v>
-      </c>
-      <c r="IB5">
-        <v>6.6795526372382397E-3</v>
-      </c>
-      <c r="IC5">
-        <v>6.7614725974346201E-3</v>
-      </c>
-      <c r="ID5">
-        <v>6.7410969877561098E-3</v>
-      </c>
-      <c r="IE5">
-        <v>6.3102392388619203E-3</v>
-      </c>
-      <c r="IF5">
-        <v>8.4474307848104307E-3</v>
-      </c>
-      <c r="IG5">
-        <v>8.1742869736347607E-3</v>
-      </c>
-      <c r="IH5">
-        <v>9.1738114242806094E-3</v>
-      </c>
-      <c r="II5">
-        <v>7.8596439093180093E-3</v>
-      </c>
-      <c r="IJ5">
-        <v>7.7530150532886003E-3</v>
-      </c>
-      <c r="IK5">
-        <v>7.7912043799653096E-3</v>
-      </c>
-      <c r="IL5">
-        <v>7.4734711807585398E-3</v>
-      </c>
-      <c r="IM5">
-        <v>7.4680745341900601E-3</v>
-      </c>
-      <c r="IN5">
-        <v>7.3237803369725898E-3</v>
-      </c>
-      <c r="IO5">
-        <v>7.3375777087661296E-3</v>
-      </c>
-      <c r="IP5">
-        <v>7.3560759100139098E-3</v>
-      </c>
-      <c r="IQ5">
-        <v>7.3718892038574799E-3</v>
-      </c>
-      <c r="IR5">
-        <v>7.41700180440962E-3</v>
-      </c>
-      <c r="IS5">
-        <v>7.4722176514185699E-3</v>
-      </c>
-      <c r="IT5">
-        <v>6.2093975197165798E-3</v>
-      </c>
-      <c r="IU5">
-        <v>6.3108978888065598E-3</v>
-      </c>
-      <c r="IV5">
-        <v>6.4164393752811398E-3</v>
-      </c>
-      <c r="IW5">
-        <v>6.5141811082534704E-3</v>
-      </c>
-      <c r="IX5">
-        <v>6.5703619384055202E-3</v>
-      </c>
-      <c r="IY5">
-        <v>6.64055047308561E-3</v>
-      </c>
-      <c r="IZ5">
-        <v>6.7345555746429102E-3</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8D75A12-56FE-494F-95BC-F47763DA8D7F}">
   <sheetPr>
     <tabColor theme="5" tint="-0.249977111117893"/>

</xml_diff>